<commit_message>
Rename race tabs to HD-##/SD-## abbreviations
"PA-LEG-13" -> "HD-13", "PA-STSEN-06" -> "SD-6" (state prefix kept
only if a file ever mixes multiple states, same disambiguation rule
as the Summary tab's friendly labels). Sheet names, cross-sheet
formula references, and Summary hyperlinks all derive from a single
race->tab-name mapping now, so they can't drift out of sync.

Left each race tab's own in-sheet header showing the raw race code
for now (e.g. "PA-LEG-13") — only the clickable tab name changed,
since that's what was asked for. Happy to make the header match too
if that reads as inconsistent in practice.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MLDJZYpWcKSroEnjKzk6cV
</commit_message>
<xml_diff>
--- a/reports/PA_Digital_Competitive_Report.xlsx
+++ b/reports/PA_Digital_Competitive_Report.xlsx
@@ -9,54 +9,54 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="PA-LEG-13" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="PA-LEG-16" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="PA-LEG-18" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="PA-LEG-28" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="PA-LEG-41" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="PA-LEG-44" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="PA-LEG-46" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="PA-LEG-72" sheetId="9" state="visible" r:id="rId11"/>
-    <sheet name="PA-LEG-88" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="PA-LEG-118" sheetId="11" state="visible" r:id="rId13"/>
-    <sheet name="PA-LEG-121" sheetId="12" state="visible" r:id="rId14"/>
-    <sheet name="PA-LEG-137" sheetId="13" state="visible" r:id="rId15"/>
-    <sheet name="PA-LEG-142" sheetId="14" state="visible" r:id="rId16"/>
-    <sheet name="PA-LEG-143" sheetId="15" state="visible" r:id="rId17"/>
-    <sheet name="PA-LEG-144" sheetId="16" state="visible" r:id="rId18"/>
-    <sheet name="PA-LEG-147" sheetId="17" state="visible" r:id="rId19"/>
-    <sheet name="PA-LEG-160" sheetId="18" state="visible" r:id="rId20"/>
-    <sheet name="PA-LEG-170" sheetId="19" state="visible" r:id="rId21"/>
-    <sheet name="PA-LEG-187" sheetId="20" state="visible" r:id="rId22"/>
-    <sheet name="PA-STSEN-06" sheetId="21" state="visible" r:id="rId23"/>
-    <sheet name="PA-STSEN-16" sheetId="22" state="visible" r:id="rId24"/>
-    <sheet name="PA-STSEN-24" sheetId="23" state="visible" r:id="rId25"/>
-    <sheet name="PA-STSEN-40" sheetId="24" state="visible" r:id="rId26"/>
+    <sheet name="HD-13" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="HD-16" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="HD-18" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="HD-28" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="HD-41" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="HD-44" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="HD-46" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="HD-72" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="HD-88" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="HD-118" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="HD-121" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="HD-137" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="HD-142" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="HD-143" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="HD-144" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="HD-147" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="HD-160" sheetId="18" state="visible" r:id="rId20"/>
+    <sheet name="HD-170" sheetId="19" state="visible" r:id="rId21"/>
+    <sheet name="HD-187" sheetId="20" state="visible" r:id="rId22"/>
+    <sheet name="SD-6" sheetId="21" state="visible" r:id="rId23"/>
+    <sheet name="SD-16" sheetId="22" state="visible" r:id="rId24"/>
+    <sheet name="SD-24" sheetId="23" state="visible" r:id="rId25"/>
+    <sheet name="SD-40" sheetId="24" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-118'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-121'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-13'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-137'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-142'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="14" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-143'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="15" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-144'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="16" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-147'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-16'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="17" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-160'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="18" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-170'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-18'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="19" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-187'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-28'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-41'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-44'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-46'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-72'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Titles" vbProcedure="false">'PA-LEG-88'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="20" name="_xlnm.Print_Titles" vbProcedure="false">'PA-STSEN-06'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="21" name="_xlnm.Print_Titles" vbProcedure="false">'PA-STSEN-16'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="22" name="_xlnm.Print_Titles" vbProcedure="false">'PA-STSEN-24'!$1:$3</definedName>
-    <definedName function="false" hidden="false" localSheetId="23" name="_xlnm.Print_Titles" vbProcedure="false">'PA-STSEN-40'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="10" name="_xlnm.Print_Titles" vbProcedure="false">'HD-118'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="11" name="_xlnm.Print_Titles" vbProcedure="false">'HD-121'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'HD-13'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="12" name="_xlnm.Print_Titles" vbProcedure="false">'HD-137'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="13" name="_xlnm.Print_Titles" vbProcedure="false">'HD-142'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="14" name="_xlnm.Print_Titles" vbProcedure="false">'HD-143'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="15" name="_xlnm.Print_Titles" vbProcedure="false">'HD-144'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="16" name="_xlnm.Print_Titles" vbProcedure="false">'HD-147'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">'HD-16'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="17" name="_xlnm.Print_Titles" vbProcedure="false">'HD-160'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="18" name="_xlnm.Print_Titles" vbProcedure="false">'HD-170'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">'HD-18'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="19" name="_xlnm.Print_Titles" vbProcedure="false">'HD-187'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">'HD-28'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Titles" vbProcedure="false">'HD-41'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Titles" vbProcedure="false">'HD-44'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Titles" vbProcedure="false">'HD-46'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Titles" vbProcedure="false">'HD-72'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Titles" vbProcedure="false">'HD-88'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="21" name="_xlnm.Print_Titles" vbProcedure="false">'SD-16'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="22" name="_xlnm.Print_Titles" vbProcedure="false">'SD-24'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="23" name="_xlnm.Print_Titles" vbProcedure="false">'SD-40'!$1:$3</definedName>
+    <definedName function="false" hidden="false" localSheetId="20" name="_xlnm.Print_Titles" vbProcedure="false">'SD-6'!$1:$3</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Summary!$1:$3</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -2114,15 +2114,15 @@
         <v>8</v>
       </c>
       <c r="C4" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-13'!D$4:D$10,'PA-LEG-13'!$C$4:$C$10,"CTV")</f>
+        <f aca="false">SUMIFS('HD-13'!D$4:D$10,'HD-13'!$C$4:$C$10,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D4" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-13'!D$4:D$10,'PA-LEG-13'!$C$4:$C$10,"CTV",'PA-LEG-13'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-13'!D$4:D$10,'HD-13'!$C$4:$C$10,"CTV",'HD-13'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E4" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-13'!D$4:D$10,'PA-LEG-13'!$C$4:$C$10,"CTV",'PA-LEG-13'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-13'!D$4:D$10,'HD-13'!$C$4:$C$10,"CTV",'HD-13'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F4" s="5" t="n">
@@ -2136,15 +2136,15 @@
         <v>9</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-13'!D$4:D$10,'PA-LEG-13'!$C$4:$C$10,"Google")</f>
+        <f aca="false">SUMIFS('HD-13'!D$4:D$10,'HD-13'!$C$4:$C$10,"Google")</f>
         <v>7415.48</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-13'!D$4:D$10,'PA-LEG-13'!$C$4:$C$10,"Google",'PA-LEG-13'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-13'!D$4:D$10,'HD-13'!$C$4:$C$10,"Google",'HD-13'!$B$4:$B$10,"R")</f>
         <v>7415.48</v>
       </c>
       <c r="E5" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-13'!D$4:D$10,'PA-LEG-13'!$C$4:$C$10,"Google",'PA-LEG-13'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-13'!D$4:D$10,'HD-13'!$C$4:$C$10,"Google",'HD-13'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F5" s="5" t="n">
@@ -2158,15 +2158,15 @@
         <v>10</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-13'!D$4:D$10,'PA-LEG-13'!$C$4:$C$10,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-13'!D$4:D$10,'HD-13'!$C$4:$C$10,"Facebook")</f>
         <v>954.09</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-13'!D$4:D$10,'PA-LEG-13'!$C$4:$C$10,"Facebook",'PA-LEG-13'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-13'!D$4:D$10,'HD-13'!$C$4:$C$10,"Facebook",'HD-13'!$B$4:$B$10,"R")</f>
         <v>954.09</v>
       </c>
       <c r="E6" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-13'!D$4:D$10,'PA-LEG-13'!$C$4:$C$10,"Facebook",'PA-LEG-13'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-13'!D$4:D$10,'HD-13'!$C$4:$C$10,"Facebook",'HD-13'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F6" s="5" t="n">
@@ -2180,11 +2180,11 @@
         <v>11</v>
       </c>
       <c r="C7" s="7" t="n">
-        <f aca="false">'PA-LEG-13'!D10</f>
+        <f aca="false">'HD-13'!D10</f>
         <v>8369.57</v>
       </c>
       <c r="D7" s="7" t="n">
-        <f aca="false">'PA-LEG-13'!D8</f>
+        <f aca="false">'HD-13'!D8</f>
         <v>8369.57</v>
       </c>
       <c r="E7" s="7" t="n">
@@ -2204,15 +2204,15 @@
         <v>8</v>
       </c>
       <c r="C9" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-16'!D$4:D$12,'PA-LEG-16'!$C$4:$C$12,"CTV")</f>
+        <f aca="false">SUMIFS('HD-16'!D$4:D$12,'HD-16'!$C$4:$C$12,"CTV")</f>
         <v>510.91</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-16'!D$4:D$12,'PA-LEG-16'!$C$4:$C$12,"CTV",'PA-LEG-16'!$B$4:$B$12,"R")</f>
+        <f aca="false">SUMIFS('HD-16'!D$4:D$12,'HD-16'!$C$4:$C$12,"CTV",'HD-16'!$B$4:$B$12,"R")</f>
         <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-16'!D$4:D$12,'PA-LEG-16'!$C$4:$C$12,"CTV",'PA-LEG-16'!$B$4:$B$12,"D")</f>
+        <f aca="false">SUMIFS('HD-16'!D$4:D$12,'HD-16'!$C$4:$C$12,"CTV",'HD-16'!$B$4:$B$12,"D")</f>
         <v>510.91</v>
       </c>
       <c r="F9" s="5" t="n">
@@ -2226,15 +2226,15 @@
         <v>9</v>
       </c>
       <c r="C10" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-16'!D$4:D$12,'PA-LEG-16'!$C$4:$C$12,"Google")</f>
+        <f aca="false">SUMIFS('HD-16'!D$4:D$12,'HD-16'!$C$4:$C$12,"Google")</f>
         <v>0</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-16'!D$4:D$12,'PA-LEG-16'!$C$4:$C$12,"Google",'PA-LEG-16'!$B$4:$B$12,"R")</f>
+        <f aca="false">SUMIFS('HD-16'!D$4:D$12,'HD-16'!$C$4:$C$12,"Google",'HD-16'!$B$4:$B$12,"R")</f>
         <v>0</v>
       </c>
       <c r="E10" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-16'!D$4:D$12,'PA-LEG-16'!$C$4:$C$12,"Google",'PA-LEG-16'!$B$4:$B$12,"D")</f>
+        <f aca="false">SUMIFS('HD-16'!D$4:D$12,'HD-16'!$C$4:$C$12,"Google",'HD-16'!$B$4:$B$12,"D")</f>
         <v>0</v>
       </c>
       <c r="F10" s="5" t="n">
@@ -2248,15 +2248,15 @@
         <v>10</v>
       </c>
       <c r="C11" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-16'!D$4:D$12,'PA-LEG-16'!$C$4:$C$12,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-16'!D$4:D$12,'HD-16'!$C$4:$C$12,"Facebook")</f>
         <v>1685.02</v>
       </c>
       <c r="D11" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-16'!D$4:D$12,'PA-LEG-16'!$C$4:$C$12,"Facebook",'PA-LEG-16'!$B$4:$B$12,"R")</f>
+        <f aca="false">SUMIFS('HD-16'!D$4:D$12,'HD-16'!$C$4:$C$12,"Facebook",'HD-16'!$B$4:$B$12,"R")</f>
         <v>0</v>
       </c>
       <c r="E11" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-16'!D$4:D$12,'PA-LEG-16'!$C$4:$C$12,"Facebook",'PA-LEG-16'!$B$4:$B$12,"D")</f>
+        <f aca="false">SUMIFS('HD-16'!D$4:D$12,'HD-16'!$C$4:$C$12,"Facebook",'HD-16'!$B$4:$B$12,"D")</f>
         <v>1685.02</v>
       </c>
       <c r="F11" s="5" t="n">
@@ -2270,7 +2270,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="7" t="n">
-        <f aca="false">'PA-LEG-16'!D12</f>
+        <f aca="false">'HD-16'!D12</f>
         <v>2195.93</v>
       </c>
       <c r="D12" s="7" t="n">
@@ -2278,7 +2278,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="7" t="n">
-        <f aca="false">'PA-LEG-16'!D10</f>
+        <f aca="false">'HD-16'!D10</f>
         <v>2195.93</v>
       </c>
       <c r="F12" s="7" t="n">
@@ -2294,15 +2294,15 @@
         <v>8</v>
       </c>
       <c r="C14" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-18'!D$4:D$17,'PA-LEG-18'!$C$4:$C$17,"CTV")</f>
+        <f aca="false">SUMIFS('HD-18'!D$4:D$17,'HD-18'!$C$4:$C$17,"CTV")</f>
         <v>291.25</v>
       </c>
       <c r="D14" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-18'!D$4:D$17,'PA-LEG-18'!$C$4:$C$17,"CTV",'PA-LEG-18'!$B$4:$B$17,"R")</f>
+        <f aca="false">SUMIFS('HD-18'!D$4:D$17,'HD-18'!$C$4:$C$17,"CTV",'HD-18'!$B$4:$B$17,"R")</f>
         <v>0</v>
       </c>
       <c r="E14" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-18'!D$4:D$17,'PA-LEG-18'!$C$4:$C$17,"CTV",'PA-LEG-18'!$B$4:$B$17,"D")</f>
+        <f aca="false">SUMIFS('HD-18'!D$4:D$17,'HD-18'!$C$4:$C$17,"CTV",'HD-18'!$B$4:$B$17,"D")</f>
         <v>291.25</v>
       </c>
       <c r="F14" s="5" t="n">
@@ -2316,15 +2316,15 @@
         <v>9</v>
       </c>
       <c r="C15" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-18'!D$4:D$17,'PA-LEG-18'!$C$4:$C$17,"Google")</f>
+        <f aca="false">SUMIFS('HD-18'!D$4:D$17,'HD-18'!$C$4:$C$17,"Google")</f>
         <v>8812.82</v>
       </c>
       <c r="D15" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-18'!D$4:D$17,'PA-LEG-18'!$C$4:$C$17,"Google",'PA-LEG-18'!$B$4:$B$17,"R")</f>
+        <f aca="false">SUMIFS('HD-18'!D$4:D$17,'HD-18'!$C$4:$C$17,"Google",'HD-18'!$B$4:$B$17,"R")</f>
         <v>7791.26</v>
       </c>
       <c r="E15" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-18'!D$4:D$17,'PA-LEG-18'!$C$4:$C$17,"Google",'PA-LEG-18'!$B$4:$B$17,"D")</f>
+        <f aca="false">SUMIFS('HD-18'!D$4:D$17,'HD-18'!$C$4:$C$17,"Google",'HD-18'!$B$4:$B$17,"D")</f>
         <v>1021.56</v>
       </c>
       <c r="F15" s="5" t="n">
@@ -2338,15 +2338,15 @@
         <v>10</v>
       </c>
       <c r="C16" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-18'!D$4:D$17,'PA-LEG-18'!$C$4:$C$17,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-18'!D$4:D$17,'HD-18'!$C$4:$C$17,"Facebook")</f>
         <v>2895.61</v>
       </c>
       <c r="D16" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-18'!D$4:D$17,'PA-LEG-18'!$C$4:$C$17,"Facebook",'PA-LEG-18'!$B$4:$B$17,"R")</f>
+        <f aca="false">SUMIFS('HD-18'!D$4:D$17,'HD-18'!$C$4:$C$17,"Facebook",'HD-18'!$B$4:$B$17,"R")</f>
         <v>955.43</v>
       </c>
       <c r="E16" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-18'!D$4:D$17,'PA-LEG-18'!$C$4:$C$17,"Facebook",'PA-LEG-18'!$B$4:$B$17,"D")</f>
+        <f aca="false">SUMIFS('HD-18'!D$4:D$17,'HD-18'!$C$4:$C$17,"Facebook",'HD-18'!$B$4:$B$17,"D")</f>
         <v>1940.18</v>
       </c>
       <c r="F16" s="5" t="n">
@@ -2360,15 +2360,15 @@
         <v>11</v>
       </c>
       <c r="C17" s="7" t="n">
-        <f aca="false">'PA-LEG-18'!D17</f>
+        <f aca="false">'HD-18'!D17</f>
         <v>11999.68</v>
       </c>
       <c r="D17" s="7" t="n">
-        <f aca="false">'PA-LEG-18'!D8</f>
+        <f aca="false">'HD-18'!D8</f>
         <v>8746.69</v>
       </c>
       <c r="E17" s="7" t="n">
-        <f aca="false">'PA-LEG-18'!D15</f>
+        <f aca="false">'HD-18'!D15</f>
         <v>3252.99</v>
       </c>
       <c r="F17" s="7" t="n">
@@ -2384,15 +2384,15 @@
         <v>8</v>
       </c>
       <c r="C19" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-28'!D$4:D$10,'PA-LEG-28'!$C$4:$C$10,"CTV")</f>
+        <f aca="false">SUMIFS('HD-28'!D$4:D$10,'HD-28'!$C$4:$C$10,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-28'!D$4:D$10,'PA-LEG-28'!$C$4:$C$10,"CTV",'PA-LEG-28'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-28'!D$4:D$10,'HD-28'!$C$4:$C$10,"CTV",'HD-28'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E19" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-28'!D$4:D$10,'PA-LEG-28'!$C$4:$C$10,"CTV",'PA-LEG-28'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-28'!D$4:D$10,'HD-28'!$C$4:$C$10,"CTV",'HD-28'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F19" s="5" t="n">
@@ -2406,15 +2406,15 @@
         <v>9</v>
       </c>
       <c r="C20" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-28'!D$4:D$10,'PA-LEG-28'!$C$4:$C$10,"Google")</f>
+        <f aca="false">SUMIFS('HD-28'!D$4:D$10,'HD-28'!$C$4:$C$10,"Google")</f>
         <v>9958.28</v>
       </c>
       <c r="D20" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-28'!D$4:D$10,'PA-LEG-28'!$C$4:$C$10,"Google",'PA-LEG-28'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-28'!D$4:D$10,'HD-28'!$C$4:$C$10,"Google",'HD-28'!$B$4:$B$10,"R")</f>
         <v>9958.28</v>
       </c>
       <c r="E20" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-28'!D$4:D$10,'PA-LEG-28'!$C$4:$C$10,"Google",'PA-LEG-28'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-28'!D$4:D$10,'HD-28'!$C$4:$C$10,"Google",'HD-28'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F20" s="5" t="n">
@@ -2428,15 +2428,15 @@
         <v>10</v>
       </c>
       <c r="C21" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-28'!D$4:D$10,'PA-LEG-28'!$C$4:$C$10,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-28'!D$4:D$10,'HD-28'!$C$4:$C$10,"Facebook")</f>
         <v>1908.57</v>
       </c>
       <c r="D21" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-28'!D$4:D$10,'PA-LEG-28'!$C$4:$C$10,"Facebook",'PA-LEG-28'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-28'!D$4:D$10,'HD-28'!$C$4:$C$10,"Facebook",'HD-28'!$B$4:$B$10,"R")</f>
         <v>1908.57</v>
       </c>
       <c r="E21" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-28'!D$4:D$10,'PA-LEG-28'!$C$4:$C$10,"Facebook",'PA-LEG-28'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-28'!D$4:D$10,'HD-28'!$C$4:$C$10,"Facebook",'HD-28'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F21" s="5" t="n">
@@ -2450,11 +2450,11 @@
         <v>11</v>
       </c>
       <c r="C22" s="7" t="n">
-        <f aca="false">'PA-LEG-28'!D10</f>
+        <f aca="false">'HD-28'!D10</f>
         <v>11866.85</v>
       </c>
       <c r="D22" s="7" t="n">
-        <f aca="false">'PA-LEG-28'!D8</f>
+        <f aca="false">'HD-28'!D8</f>
         <v>11866.85</v>
       </c>
       <c r="E22" s="7" t="n">
@@ -2474,15 +2474,15 @@
         <v>8</v>
       </c>
       <c r="C24" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-41'!D$4:D$10,'PA-LEG-41'!$C$4:$C$10,"CTV")</f>
+        <f aca="false">SUMIFS('HD-41'!D$4:D$10,'HD-41'!$C$4:$C$10,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D24" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-41'!D$4:D$10,'PA-LEG-41'!$C$4:$C$10,"CTV",'PA-LEG-41'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-41'!D$4:D$10,'HD-41'!$C$4:$C$10,"CTV",'HD-41'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E24" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-41'!D$4:D$10,'PA-LEG-41'!$C$4:$C$10,"CTV",'PA-LEG-41'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-41'!D$4:D$10,'HD-41'!$C$4:$C$10,"CTV",'HD-41'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F24" s="5" t="n">
@@ -2496,15 +2496,15 @@
         <v>9</v>
       </c>
       <c r="C25" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-41'!D$4:D$10,'PA-LEG-41'!$C$4:$C$10,"Google")</f>
+        <f aca="false">SUMIFS('HD-41'!D$4:D$10,'HD-41'!$C$4:$C$10,"Google")</f>
         <v>7899.44</v>
       </c>
       <c r="D25" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-41'!D$4:D$10,'PA-LEG-41'!$C$4:$C$10,"Google",'PA-LEG-41'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-41'!D$4:D$10,'HD-41'!$C$4:$C$10,"Google",'HD-41'!$B$4:$B$10,"R")</f>
         <v>7899.44</v>
       </c>
       <c r="E25" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-41'!D$4:D$10,'PA-LEG-41'!$C$4:$C$10,"Google",'PA-LEG-41'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-41'!D$4:D$10,'HD-41'!$C$4:$C$10,"Google",'HD-41'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F25" s="5" t="n">
@@ -2518,15 +2518,15 @@
         <v>10</v>
       </c>
       <c r="C26" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-41'!D$4:D$10,'PA-LEG-41'!$C$4:$C$10,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-41'!D$4:D$10,'HD-41'!$C$4:$C$10,"Facebook")</f>
         <v>901.12</v>
       </c>
       <c r="D26" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-41'!D$4:D$10,'PA-LEG-41'!$C$4:$C$10,"Facebook",'PA-LEG-41'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-41'!D$4:D$10,'HD-41'!$C$4:$C$10,"Facebook",'HD-41'!$B$4:$B$10,"R")</f>
         <v>901.12</v>
       </c>
       <c r="E26" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-41'!D$4:D$10,'PA-LEG-41'!$C$4:$C$10,"Facebook",'PA-LEG-41'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-41'!D$4:D$10,'HD-41'!$C$4:$C$10,"Facebook",'HD-41'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F26" s="5" t="n">
@@ -2540,11 +2540,11 @@
         <v>11</v>
       </c>
       <c r="C27" s="7" t="n">
-        <f aca="false">'PA-LEG-41'!D10</f>
+        <f aca="false">'HD-41'!D10</f>
         <v>8800.56</v>
       </c>
       <c r="D27" s="7" t="n">
-        <f aca="false">'PA-LEG-41'!D8</f>
+        <f aca="false">'HD-41'!D8</f>
         <v>8800.56</v>
       </c>
       <c r="E27" s="7" t="n">
@@ -2564,15 +2564,15 @@
         <v>8</v>
       </c>
       <c r="C29" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-44'!D$4:D$23,'PA-LEG-44'!$C$4:$C$23,"CTV")</f>
+        <f aca="false">SUMIFS('HD-44'!D$4:D$23,'HD-44'!$C$4:$C$23,"CTV")</f>
         <v>985.79</v>
       </c>
       <c r="D29" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-44'!D$4:D$23,'PA-LEG-44'!$C$4:$C$23,"CTV",'PA-LEG-44'!$B$4:$B$23,"R")</f>
+        <f aca="false">SUMIFS('HD-44'!D$4:D$23,'HD-44'!$C$4:$C$23,"CTV",'HD-44'!$B$4:$B$23,"R")</f>
         <v>0</v>
       </c>
       <c r="E29" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-44'!D$4:D$23,'PA-LEG-44'!$C$4:$C$23,"CTV",'PA-LEG-44'!$B$4:$B$23,"D")</f>
+        <f aca="false">SUMIFS('HD-44'!D$4:D$23,'HD-44'!$C$4:$C$23,"CTV",'HD-44'!$B$4:$B$23,"D")</f>
         <v>985.79</v>
       </c>
       <c r="F29" s="5" t="n">
@@ -2586,15 +2586,15 @@
         <v>9</v>
       </c>
       <c r="C30" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-44'!D$4:D$23,'PA-LEG-44'!$C$4:$C$23,"Google")</f>
+        <f aca="false">SUMIFS('HD-44'!D$4:D$23,'HD-44'!$C$4:$C$23,"Google")</f>
         <v>13026.89</v>
       </c>
       <c r="D30" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-44'!D$4:D$23,'PA-LEG-44'!$C$4:$C$23,"Google",'PA-LEG-44'!$B$4:$B$23,"R")</f>
+        <f aca="false">SUMIFS('HD-44'!D$4:D$23,'HD-44'!$C$4:$C$23,"Google",'HD-44'!$B$4:$B$23,"R")</f>
         <v>9522.05</v>
       </c>
       <c r="E30" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-44'!D$4:D$23,'PA-LEG-44'!$C$4:$C$23,"Google",'PA-LEG-44'!$B$4:$B$23,"D")</f>
+        <f aca="false">SUMIFS('HD-44'!D$4:D$23,'HD-44'!$C$4:$C$23,"Google",'HD-44'!$B$4:$B$23,"D")</f>
         <v>3504.84</v>
       </c>
       <c r="F30" s="5" t="n">
@@ -2608,15 +2608,15 @@
         <v>10</v>
       </c>
       <c r="C31" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-44'!D$4:D$23,'PA-LEG-44'!$C$4:$C$23,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-44'!D$4:D$23,'HD-44'!$C$4:$C$23,"Facebook")</f>
         <v>6641.09</v>
       </c>
       <c r="D31" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-44'!D$4:D$23,'PA-LEG-44'!$C$4:$C$23,"Facebook",'PA-LEG-44'!$B$4:$B$23,"R")</f>
+        <f aca="false">SUMIFS('HD-44'!D$4:D$23,'HD-44'!$C$4:$C$23,"Facebook",'HD-44'!$B$4:$B$23,"R")</f>
         <v>1592.3</v>
       </c>
       <c r="E31" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-44'!D$4:D$23,'PA-LEG-44'!$C$4:$C$23,"Facebook",'PA-LEG-44'!$B$4:$B$23,"D")</f>
+        <f aca="false">SUMIFS('HD-44'!D$4:D$23,'HD-44'!$C$4:$C$23,"Facebook",'HD-44'!$B$4:$B$23,"D")</f>
         <v>5048.79</v>
       </c>
       <c r="F31" s="5" t="n">
@@ -2630,15 +2630,15 @@
         <v>11</v>
       </c>
       <c r="C32" s="7" t="n">
-        <f aca="false">'PA-LEG-44'!D23</f>
+        <f aca="false">'HD-44'!D23</f>
         <v>20653.77</v>
       </c>
       <c r="D32" s="7" t="n">
-        <f aca="false">'PA-LEG-44'!D8</f>
+        <f aca="false">'HD-44'!D8</f>
         <v>11114.35</v>
       </c>
       <c r="E32" s="7" t="n">
-        <f aca="false">'PA-LEG-44'!D21</f>
+        <f aca="false">'HD-44'!D21</f>
         <v>9539.42</v>
       </c>
       <c r="F32" s="7" t="n">
@@ -2654,15 +2654,15 @@
         <v>8</v>
       </c>
       <c r="C34" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-46'!D$4:D$10,'PA-LEG-46'!$C$4:$C$10,"CTV")</f>
+        <f aca="false">SUMIFS('HD-46'!D$4:D$10,'HD-46'!$C$4:$C$10,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D34" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-46'!D$4:D$10,'PA-LEG-46'!$C$4:$C$10,"CTV",'PA-LEG-46'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-46'!D$4:D$10,'HD-46'!$C$4:$C$10,"CTV",'HD-46'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E34" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-46'!D$4:D$10,'PA-LEG-46'!$C$4:$C$10,"CTV",'PA-LEG-46'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-46'!D$4:D$10,'HD-46'!$C$4:$C$10,"CTV",'HD-46'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F34" s="5" t="n">
@@ -2676,15 +2676,15 @@
         <v>9</v>
       </c>
       <c r="C35" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-46'!D$4:D$10,'PA-LEG-46'!$C$4:$C$10,"Google")</f>
+        <f aca="false">SUMIFS('HD-46'!D$4:D$10,'HD-46'!$C$4:$C$10,"Google")</f>
         <v>600</v>
       </c>
       <c r="D35" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-46'!D$4:D$10,'PA-LEG-46'!$C$4:$C$10,"Google",'PA-LEG-46'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-46'!D$4:D$10,'HD-46'!$C$4:$C$10,"Google",'HD-46'!$B$4:$B$10,"R")</f>
         <v>600</v>
       </c>
       <c r="E35" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-46'!D$4:D$10,'PA-LEG-46'!$C$4:$C$10,"Google",'PA-LEG-46'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-46'!D$4:D$10,'HD-46'!$C$4:$C$10,"Google",'HD-46'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F35" s="5" t="n">
@@ -2698,15 +2698,15 @@
         <v>10</v>
       </c>
       <c r="C36" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-46'!D$4:D$10,'PA-LEG-46'!$C$4:$C$10,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-46'!D$4:D$10,'HD-46'!$C$4:$C$10,"Facebook")</f>
         <v>1140.3</v>
       </c>
       <c r="D36" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-46'!D$4:D$10,'PA-LEG-46'!$C$4:$C$10,"Facebook",'PA-LEG-46'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-46'!D$4:D$10,'HD-46'!$C$4:$C$10,"Facebook",'HD-46'!$B$4:$B$10,"R")</f>
         <v>1140.3</v>
       </c>
       <c r="E36" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-46'!D$4:D$10,'PA-LEG-46'!$C$4:$C$10,"Facebook",'PA-LEG-46'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-46'!D$4:D$10,'HD-46'!$C$4:$C$10,"Facebook",'HD-46'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F36" s="5" t="n">
@@ -2720,11 +2720,11 @@
         <v>11</v>
       </c>
       <c r="C37" s="7" t="n">
-        <f aca="false">'PA-LEG-46'!D10</f>
+        <f aca="false">'HD-46'!D10</f>
         <v>1740.3</v>
       </c>
       <c r="D37" s="7" t="n">
-        <f aca="false">'PA-LEG-46'!D8</f>
+        <f aca="false">'HD-46'!D8</f>
         <v>1740.3</v>
       </c>
       <c r="E37" s="7" t="n">
@@ -2744,15 +2744,15 @@
         <v>8</v>
       </c>
       <c r="C39" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-72'!D$4:D$26,'PA-LEG-72'!$C$4:$C$26,"CTV")</f>
+        <f aca="false">SUMIFS('HD-72'!D$4:D$26,'HD-72'!$C$4:$C$26,"CTV")</f>
         <v>67673.63</v>
       </c>
       <c r="D39" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-72'!D$4:D$26,'PA-LEG-72'!$C$4:$C$26,"CTV",'PA-LEG-72'!$B$4:$B$26,"R")</f>
+        <f aca="false">SUMIFS('HD-72'!D$4:D$26,'HD-72'!$C$4:$C$26,"CTV",'HD-72'!$B$4:$B$26,"R")</f>
         <v>0</v>
       </c>
       <c r="E39" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-72'!D$4:D$26,'PA-LEG-72'!$C$4:$C$26,"CTV",'PA-LEG-72'!$B$4:$B$26,"D")</f>
+        <f aca="false">SUMIFS('HD-72'!D$4:D$26,'HD-72'!$C$4:$C$26,"CTV",'HD-72'!$B$4:$B$26,"D")</f>
         <v>67673.63</v>
       </c>
       <c r="F39" s="5" t="n">
@@ -2766,15 +2766,15 @@
         <v>9</v>
       </c>
       <c r="C40" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-72'!D$4:D$26,'PA-LEG-72'!$C$4:$C$26,"Google")</f>
+        <f aca="false">SUMIFS('HD-72'!D$4:D$26,'HD-72'!$C$4:$C$26,"Google")</f>
         <v>22139.3</v>
       </c>
       <c r="D40" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-72'!D$4:D$26,'PA-LEG-72'!$C$4:$C$26,"Google",'PA-LEG-72'!$B$4:$B$26,"R")</f>
+        <f aca="false">SUMIFS('HD-72'!D$4:D$26,'HD-72'!$C$4:$C$26,"Google",'HD-72'!$B$4:$B$26,"R")</f>
         <v>19315.89</v>
       </c>
       <c r="E40" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-72'!D$4:D$26,'PA-LEG-72'!$C$4:$C$26,"Google",'PA-LEG-72'!$B$4:$B$26,"D")</f>
+        <f aca="false">SUMIFS('HD-72'!D$4:D$26,'HD-72'!$C$4:$C$26,"Google",'HD-72'!$B$4:$B$26,"D")</f>
         <v>2823.41</v>
       </c>
       <c r="F40" s="5" t="n">
@@ -2788,15 +2788,15 @@
         <v>10</v>
       </c>
       <c r="C41" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-72'!D$4:D$26,'PA-LEG-72'!$C$4:$C$26,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-72'!D$4:D$26,'HD-72'!$C$4:$C$26,"Facebook")</f>
         <v>11303.9</v>
       </c>
       <c r="D41" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-72'!D$4:D$26,'PA-LEG-72'!$C$4:$C$26,"Facebook",'PA-LEG-72'!$B$4:$B$26,"R")</f>
+        <f aca="false">SUMIFS('HD-72'!D$4:D$26,'HD-72'!$C$4:$C$26,"Facebook",'HD-72'!$B$4:$B$26,"R")</f>
         <v>1656.18</v>
       </c>
       <c r="E41" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-72'!D$4:D$26,'PA-LEG-72'!$C$4:$C$26,"Facebook",'PA-LEG-72'!$B$4:$B$26,"D")</f>
+        <f aca="false">SUMIFS('HD-72'!D$4:D$26,'HD-72'!$C$4:$C$26,"Facebook",'HD-72'!$B$4:$B$26,"D")</f>
         <v>9647.72</v>
       </c>
       <c r="F41" s="5" t="n">
@@ -2810,15 +2810,15 @@
         <v>11</v>
       </c>
       <c r="C42" s="7" t="n">
-        <f aca="false">'PA-LEG-72'!D26</f>
+        <f aca="false">'HD-72'!D26</f>
         <v>101116.83</v>
       </c>
       <c r="D42" s="7" t="n">
-        <f aca="false">'PA-LEG-72'!D11</f>
+        <f aca="false">'HD-72'!D11</f>
         <v>20972.07</v>
       </c>
       <c r="E42" s="7" t="n">
-        <f aca="false">'PA-LEG-72'!D24</f>
+        <f aca="false">'HD-72'!D24</f>
         <v>80144.76</v>
       </c>
       <c r="F42" s="7" t="n">
@@ -2834,15 +2834,15 @@
         <v>8</v>
       </c>
       <c r="C44" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-88'!D$4:D$15,'PA-LEG-88'!$C$4:$C$15,"CTV")</f>
+        <f aca="false">SUMIFS('HD-88'!D$4:D$15,'HD-88'!$C$4:$C$15,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D44" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-88'!D$4:D$15,'PA-LEG-88'!$C$4:$C$15,"CTV",'PA-LEG-88'!$B$4:$B$15,"R")</f>
+        <f aca="false">SUMIFS('HD-88'!D$4:D$15,'HD-88'!$C$4:$C$15,"CTV",'HD-88'!$B$4:$B$15,"R")</f>
         <v>0</v>
       </c>
       <c r="E44" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-88'!D$4:D$15,'PA-LEG-88'!$C$4:$C$15,"CTV",'PA-LEG-88'!$B$4:$B$15,"D")</f>
+        <f aca="false">SUMIFS('HD-88'!D$4:D$15,'HD-88'!$C$4:$C$15,"CTV",'HD-88'!$B$4:$B$15,"D")</f>
         <v>0</v>
       </c>
       <c r="F44" s="5" t="n">
@@ -2856,15 +2856,15 @@
         <v>9</v>
       </c>
       <c r="C45" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-88'!D$4:D$15,'PA-LEG-88'!$C$4:$C$15,"Google")</f>
+        <f aca="false">SUMIFS('HD-88'!D$4:D$15,'HD-88'!$C$4:$C$15,"Google")</f>
         <v>8032.72</v>
       </c>
       <c r="D45" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-88'!D$4:D$15,'PA-LEG-88'!$C$4:$C$15,"Google",'PA-LEG-88'!$B$4:$B$15,"R")</f>
+        <f aca="false">SUMIFS('HD-88'!D$4:D$15,'HD-88'!$C$4:$C$15,"Google",'HD-88'!$B$4:$B$15,"R")</f>
         <v>8032.72</v>
       </c>
       <c r="E45" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-88'!D$4:D$15,'PA-LEG-88'!$C$4:$C$15,"Google",'PA-LEG-88'!$B$4:$B$15,"D")</f>
+        <f aca="false">SUMIFS('HD-88'!D$4:D$15,'HD-88'!$C$4:$C$15,"Google",'HD-88'!$B$4:$B$15,"D")</f>
         <v>0</v>
       </c>
       <c r="F45" s="5" t="n">
@@ -2878,15 +2878,15 @@
         <v>10</v>
       </c>
       <c r="C46" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-88'!D$4:D$15,'PA-LEG-88'!$C$4:$C$15,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-88'!D$4:D$15,'HD-88'!$C$4:$C$15,"Facebook")</f>
         <v>3701.28</v>
       </c>
       <c r="D46" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-88'!D$4:D$15,'PA-LEG-88'!$C$4:$C$15,"Facebook",'PA-LEG-88'!$B$4:$B$15,"R")</f>
+        <f aca="false">SUMIFS('HD-88'!D$4:D$15,'HD-88'!$C$4:$C$15,"Facebook",'HD-88'!$B$4:$B$15,"R")</f>
         <v>672.68</v>
       </c>
       <c r="E46" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-88'!D$4:D$15,'PA-LEG-88'!$C$4:$C$15,"Facebook",'PA-LEG-88'!$B$4:$B$15,"D")</f>
+        <f aca="false">SUMIFS('HD-88'!D$4:D$15,'HD-88'!$C$4:$C$15,"Facebook",'HD-88'!$B$4:$B$15,"D")</f>
         <v>3028.6</v>
       </c>
       <c r="F46" s="5" t="n">
@@ -2900,15 +2900,15 @@
         <v>11</v>
       </c>
       <c r="C47" s="7" t="n">
-        <f aca="false">'PA-LEG-88'!D15</f>
+        <f aca="false">'HD-88'!D15</f>
         <v>11734</v>
       </c>
       <c r="D47" s="7" t="n">
-        <f aca="false">'PA-LEG-88'!D8</f>
+        <f aca="false">'HD-88'!D8</f>
         <v>8705.4</v>
       </c>
       <c r="E47" s="7" t="n">
-        <f aca="false">'PA-LEG-88'!D13</f>
+        <f aca="false">'HD-88'!D13</f>
         <v>3028.6</v>
       </c>
       <c r="F47" s="7" t="n">
@@ -2924,15 +2924,15 @@
         <v>8</v>
       </c>
       <c r="C49" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-118'!D$4:D$18,'PA-LEG-118'!$C$4:$C$18,"CTV")</f>
+        <f aca="false">SUMIFS('HD-118'!D$4:D$18,'HD-118'!$C$4:$C$18,"CTV")</f>
         <v>2510.2</v>
       </c>
       <c r="D49" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-118'!D$4:D$18,'PA-LEG-118'!$C$4:$C$18,"CTV",'PA-LEG-118'!$B$4:$B$18,"R")</f>
+        <f aca="false">SUMIFS('HD-118'!D$4:D$18,'HD-118'!$C$4:$C$18,"CTV",'HD-118'!$B$4:$B$18,"R")</f>
         <v>0</v>
       </c>
       <c r="E49" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-118'!D$4:D$18,'PA-LEG-118'!$C$4:$C$18,"CTV",'PA-LEG-118'!$B$4:$B$18,"D")</f>
+        <f aca="false">SUMIFS('HD-118'!D$4:D$18,'HD-118'!$C$4:$C$18,"CTV",'HD-118'!$B$4:$B$18,"D")</f>
         <v>2510.2</v>
       </c>
       <c r="F49" s="5" t="n">
@@ -2946,15 +2946,15 @@
         <v>9</v>
       </c>
       <c r="C50" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-118'!D$4:D$18,'PA-LEG-118'!$C$4:$C$18,"Google")</f>
+        <f aca="false">SUMIFS('HD-118'!D$4:D$18,'HD-118'!$C$4:$C$18,"Google")</f>
         <v>9883.41</v>
       </c>
       <c r="D50" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-118'!D$4:D$18,'PA-LEG-118'!$C$4:$C$18,"Google",'PA-LEG-118'!$B$4:$B$18,"R")</f>
+        <f aca="false">SUMIFS('HD-118'!D$4:D$18,'HD-118'!$C$4:$C$18,"Google",'HD-118'!$B$4:$B$18,"R")</f>
         <v>8287.54</v>
       </c>
       <c r="E50" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-118'!D$4:D$18,'PA-LEG-118'!$C$4:$C$18,"Google",'PA-LEG-118'!$B$4:$B$18,"D")</f>
+        <f aca="false">SUMIFS('HD-118'!D$4:D$18,'HD-118'!$C$4:$C$18,"Google",'HD-118'!$B$4:$B$18,"D")</f>
         <v>1595.87</v>
       </c>
       <c r="F50" s="5" t="n">
@@ -2968,15 +2968,15 @@
         <v>10</v>
       </c>
       <c r="C51" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-118'!D$4:D$18,'PA-LEG-118'!$C$4:$C$18,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-118'!D$4:D$18,'HD-118'!$C$4:$C$18,"Facebook")</f>
         <v>950.53</v>
       </c>
       <c r="D51" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-118'!D$4:D$18,'PA-LEG-118'!$C$4:$C$18,"Facebook",'PA-LEG-118'!$B$4:$B$18,"R")</f>
+        <f aca="false">SUMIFS('HD-118'!D$4:D$18,'HD-118'!$C$4:$C$18,"Facebook",'HD-118'!$B$4:$B$18,"R")</f>
         <v>950.53</v>
       </c>
       <c r="E51" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-118'!D$4:D$18,'PA-LEG-118'!$C$4:$C$18,"Facebook",'PA-LEG-118'!$B$4:$B$18,"D")</f>
+        <f aca="false">SUMIFS('HD-118'!D$4:D$18,'HD-118'!$C$4:$C$18,"Facebook",'HD-118'!$B$4:$B$18,"D")</f>
         <v>0</v>
       </c>
       <c r="F51" s="5" t="n">
@@ -2990,15 +2990,15 @@
         <v>11</v>
       </c>
       <c r="C52" s="7" t="n">
-        <f aca="false">'PA-LEG-118'!D18</f>
+        <f aca="false">'HD-118'!D18</f>
         <v>13344.14</v>
       </c>
       <c r="D52" s="7" t="n">
-        <f aca="false">'PA-LEG-118'!D8</f>
+        <f aca="false">'HD-118'!D8</f>
         <v>9238.07</v>
       </c>
       <c r="E52" s="7" t="n">
-        <f aca="false">'PA-LEG-118'!D16</f>
+        <f aca="false">'HD-118'!D16</f>
         <v>4106.07</v>
       </c>
       <c r="F52" s="7" t="n">
@@ -3014,15 +3014,15 @@
         <v>8</v>
       </c>
       <c r="C54" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-121'!D$4:D$10,'PA-LEG-121'!$C$4:$C$10,"CTV")</f>
+        <f aca="false">SUMIFS('HD-121'!D$4:D$10,'HD-121'!$C$4:$C$10,"CTV")</f>
         <v>7904.74</v>
       </c>
       <c r="D54" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-121'!D$4:D$10,'PA-LEG-121'!$C$4:$C$10,"CTV",'PA-LEG-121'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-121'!D$4:D$10,'HD-121'!$C$4:$C$10,"CTV",'HD-121'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E54" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-121'!D$4:D$10,'PA-LEG-121'!$C$4:$C$10,"CTV",'PA-LEG-121'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-121'!D$4:D$10,'HD-121'!$C$4:$C$10,"CTV",'HD-121'!$B$4:$B$10,"D")</f>
         <v>7904.74</v>
       </c>
       <c r="F54" s="5" t="n">
@@ -3036,15 +3036,15 @@
         <v>9</v>
       </c>
       <c r="C55" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-121'!D$4:D$10,'PA-LEG-121'!$C$4:$C$10,"Google")</f>
+        <f aca="false">SUMIFS('HD-121'!D$4:D$10,'HD-121'!$C$4:$C$10,"Google")</f>
         <v>15100</v>
       </c>
       <c r="D55" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-121'!D$4:D$10,'PA-LEG-121'!$C$4:$C$10,"Google",'PA-LEG-121'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-121'!D$4:D$10,'HD-121'!$C$4:$C$10,"Google",'HD-121'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E55" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-121'!D$4:D$10,'PA-LEG-121'!$C$4:$C$10,"Google",'PA-LEG-121'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-121'!D$4:D$10,'HD-121'!$C$4:$C$10,"Google",'HD-121'!$B$4:$B$10,"D")</f>
         <v>15100</v>
       </c>
       <c r="F55" s="5" t="n">
@@ -3058,15 +3058,15 @@
         <v>10</v>
       </c>
       <c r="C56" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-121'!D$4:D$10,'PA-LEG-121'!$C$4:$C$10,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-121'!D$4:D$10,'HD-121'!$C$4:$C$10,"Facebook")</f>
         <v>0</v>
       </c>
       <c r="D56" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-121'!D$4:D$10,'PA-LEG-121'!$C$4:$C$10,"Facebook",'PA-LEG-121'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-121'!D$4:D$10,'HD-121'!$C$4:$C$10,"Facebook",'HD-121'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E56" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-121'!D$4:D$10,'PA-LEG-121'!$C$4:$C$10,"Facebook",'PA-LEG-121'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-121'!D$4:D$10,'HD-121'!$C$4:$C$10,"Facebook",'HD-121'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F56" s="5" t="n">
@@ -3080,7 +3080,7 @@
         <v>11</v>
       </c>
       <c r="C57" s="7" t="n">
-        <f aca="false">'PA-LEG-121'!D10</f>
+        <f aca="false">'HD-121'!D10</f>
         <v>23004.74</v>
       </c>
       <c r="D57" s="7" t="n">
@@ -3088,7 +3088,7 @@
         <v>0</v>
       </c>
       <c r="E57" s="7" t="n">
-        <f aca="false">'PA-LEG-121'!D8</f>
+        <f aca="false">'HD-121'!D8</f>
         <v>23004.74</v>
       </c>
       <c r="F57" s="7" t="n">
@@ -3104,15 +3104,15 @@
         <v>8</v>
       </c>
       <c r="C59" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-137'!D$4:D$23,'PA-LEG-137'!$C$4:$C$23,"CTV")</f>
+        <f aca="false">SUMIFS('HD-137'!D$4:D$23,'HD-137'!$C$4:$C$23,"CTV")</f>
         <v>53763.57</v>
       </c>
       <c r="D59" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-137'!D$4:D$23,'PA-LEG-137'!$C$4:$C$23,"CTV",'PA-LEG-137'!$B$4:$B$23,"R")</f>
+        <f aca="false">SUMIFS('HD-137'!D$4:D$23,'HD-137'!$C$4:$C$23,"CTV",'HD-137'!$B$4:$B$23,"R")</f>
         <v>0</v>
       </c>
       <c r="E59" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-137'!D$4:D$23,'PA-LEG-137'!$C$4:$C$23,"CTV",'PA-LEG-137'!$B$4:$B$23,"D")</f>
+        <f aca="false">SUMIFS('HD-137'!D$4:D$23,'HD-137'!$C$4:$C$23,"CTV",'HD-137'!$B$4:$B$23,"D")</f>
         <v>53763.57</v>
       </c>
       <c r="F59" s="5" t="n">
@@ -3126,15 +3126,15 @@
         <v>9</v>
       </c>
       <c r="C60" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-137'!D$4:D$23,'PA-LEG-137'!$C$4:$C$23,"Google")</f>
+        <f aca="false">SUMIFS('HD-137'!D$4:D$23,'HD-137'!$C$4:$C$23,"Google")</f>
         <v>18841.78</v>
       </c>
       <c r="D60" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-137'!D$4:D$23,'PA-LEG-137'!$C$4:$C$23,"Google",'PA-LEG-137'!$B$4:$B$23,"R")</f>
+        <f aca="false">SUMIFS('HD-137'!D$4:D$23,'HD-137'!$C$4:$C$23,"Google",'HD-137'!$B$4:$B$23,"R")</f>
         <v>11017.23</v>
       </c>
       <c r="E60" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-137'!D$4:D$23,'PA-LEG-137'!$C$4:$C$23,"Google",'PA-LEG-137'!$B$4:$B$23,"D")</f>
+        <f aca="false">SUMIFS('HD-137'!D$4:D$23,'HD-137'!$C$4:$C$23,"Google",'HD-137'!$B$4:$B$23,"D")</f>
         <v>7824.55</v>
       </c>
       <c r="F60" s="5" t="n">
@@ -3148,15 +3148,15 @@
         <v>10</v>
       </c>
       <c r="C61" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-137'!D$4:D$23,'PA-LEG-137'!$C$4:$C$23,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-137'!D$4:D$23,'HD-137'!$C$4:$C$23,"Facebook")</f>
         <v>6365.43</v>
       </c>
       <c r="D61" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-137'!D$4:D$23,'PA-LEG-137'!$C$4:$C$23,"Facebook",'PA-LEG-137'!$B$4:$B$23,"R")</f>
+        <f aca="false">SUMIFS('HD-137'!D$4:D$23,'HD-137'!$C$4:$C$23,"Facebook",'HD-137'!$B$4:$B$23,"R")</f>
         <v>3487.41</v>
       </c>
       <c r="E61" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-137'!D$4:D$23,'PA-LEG-137'!$C$4:$C$23,"Facebook",'PA-LEG-137'!$B$4:$B$23,"D")</f>
+        <f aca="false">SUMIFS('HD-137'!D$4:D$23,'HD-137'!$C$4:$C$23,"Facebook",'HD-137'!$B$4:$B$23,"D")</f>
         <v>2878.02</v>
       </c>
       <c r="F61" s="5" t="n">
@@ -3170,15 +3170,15 @@
         <v>11</v>
       </c>
       <c r="C62" s="7" t="n">
-        <f aca="false">'PA-LEG-137'!D23</f>
+        <f aca="false">'HD-137'!D23</f>
         <v>78970.78</v>
       </c>
       <c r="D62" s="7" t="n">
-        <f aca="false">'PA-LEG-137'!D11</f>
+        <f aca="false">'HD-137'!D11</f>
         <v>14504.64</v>
       </c>
       <c r="E62" s="7" t="n">
-        <f aca="false">'PA-LEG-137'!D21</f>
+        <f aca="false">'HD-137'!D21</f>
         <v>64466.14</v>
       </c>
       <c r="F62" s="7" t="n">
@@ -3194,15 +3194,15 @@
         <v>8</v>
       </c>
       <c r="C64" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-142'!D$4:D$18,'PA-LEG-142'!$C$4:$C$18,"CTV")</f>
+        <f aca="false">SUMIFS('HD-142'!D$4:D$18,'HD-142'!$C$4:$C$18,"CTV")</f>
         <v>288.25</v>
       </c>
       <c r="D64" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-142'!D$4:D$18,'PA-LEG-142'!$C$4:$C$18,"CTV",'PA-LEG-142'!$B$4:$B$18,"R")</f>
+        <f aca="false">SUMIFS('HD-142'!D$4:D$18,'HD-142'!$C$4:$C$18,"CTV",'HD-142'!$B$4:$B$18,"R")</f>
         <v>0</v>
       </c>
       <c r="E64" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-142'!D$4:D$18,'PA-LEG-142'!$C$4:$C$18,"CTV",'PA-LEG-142'!$B$4:$B$18,"D")</f>
+        <f aca="false">SUMIFS('HD-142'!D$4:D$18,'HD-142'!$C$4:$C$18,"CTV",'HD-142'!$B$4:$B$18,"D")</f>
         <v>288.25</v>
       </c>
       <c r="F64" s="5" t="n">
@@ -3216,15 +3216,15 @@
         <v>9</v>
       </c>
       <c r="C65" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-142'!D$4:D$18,'PA-LEG-142'!$C$4:$C$18,"Google")</f>
+        <f aca="false">SUMIFS('HD-142'!D$4:D$18,'HD-142'!$C$4:$C$18,"Google")</f>
         <v>9083.11</v>
       </c>
       <c r="D65" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-142'!D$4:D$18,'PA-LEG-142'!$C$4:$C$18,"Google",'PA-LEG-142'!$B$4:$B$18,"R")</f>
+        <f aca="false">SUMIFS('HD-142'!D$4:D$18,'HD-142'!$C$4:$C$18,"Google",'HD-142'!$B$4:$B$18,"R")</f>
         <v>9083.11</v>
       </c>
       <c r="E65" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-142'!D$4:D$18,'PA-LEG-142'!$C$4:$C$18,"Google",'PA-LEG-142'!$B$4:$B$18,"D")</f>
+        <f aca="false">SUMIFS('HD-142'!D$4:D$18,'HD-142'!$C$4:$C$18,"Google",'HD-142'!$B$4:$B$18,"D")</f>
         <v>0</v>
       </c>
       <c r="F65" s="5" t="n">
@@ -3238,15 +3238,15 @@
         <v>10</v>
       </c>
       <c r="C66" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-142'!D$4:D$18,'PA-LEG-142'!$C$4:$C$18,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-142'!D$4:D$18,'HD-142'!$C$4:$C$18,"Facebook")</f>
         <v>4120.32</v>
       </c>
       <c r="D66" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-142'!D$4:D$18,'PA-LEG-142'!$C$4:$C$18,"Facebook",'PA-LEG-142'!$B$4:$B$18,"R")</f>
+        <f aca="false">SUMIFS('HD-142'!D$4:D$18,'HD-142'!$C$4:$C$18,"Facebook",'HD-142'!$B$4:$B$18,"R")</f>
         <v>1153.65</v>
       </c>
       <c r="E66" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-142'!D$4:D$18,'PA-LEG-142'!$C$4:$C$18,"Facebook",'PA-LEG-142'!$B$4:$B$18,"D")</f>
+        <f aca="false">SUMIFS('HD-142'!D$4:D$18,'HD-142'!$C$4:$C$18,"Facebook",'HD-142'!$B$4:$B$18,"D")</f>
         <v>2966.67</v>
       </c>
       <c r="F66" s="5" t="n">
@@ -3260,15 +3260,15 @@
         <v>11</v>
       </c>
       <c r="C67" s="7" t="n">
-        <f aca="false">'PA-LEG-142'!D18</f>
+        <f aca="false">'HD-142'!D18</f>
         <v>13491.68</v>
       </c>
       <c r="D67" s="7" t="n">
-        <f aca="false">'PA-LEG-142'!D8</f>
+        <f aca="false">'HD-142'!D8</f>
         <v>10236.76</v>
       </c>
       <c r="E67" s="7" t="n">
-        <f aca="false">'PA-LEG-142'!D16</f>
+        <f aca="false">'HD-142'!D16</f>
         <v>3254.92</v>
       </c>
       <c r="F67" s="7" t="n">
@@ -3284,15 +3284,15 @@
         <v>8</v>
       </c>
       <c r="C69" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-143'!D$4:D$10,'PA-LEG-143'!$C$4:$C$10,"CTV")</f>
+        <f aca="false">SUMIFS('HD-143'!D$4:D$10,'HD-143'!$C$4:$C$10,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D69" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-143'!D$4:D$10,'PA-LEG-143'!$C$4:$C$10,"CTV",'PA-LEG-143'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-143'!D$4:D$10,'HD-143'!$C$4:$C$10,"CTV",'HD-143'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E69" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-143'!D$4:D$10,'PA-LEG-143'!$C$4:$C$10,"CTV",'PA-LEG-143'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-143'!D$4:D$10,'HD-143'!$C$4:$C$10,"CTV",'HD-143'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F69" s="5" t="n">
@@ -3306,15 +3306,15 @@
         <v>9</v>
       </c>
       <c r="C70" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-143'!D$4:D$10,'PA-LEG-143'!$C$4:$C$10,"Google")</f>
+        <f aca="false">SUMIFS('HD-143'!D$4:D$10,'HD-143'!$C$4:$C$10,"Google")</f>
         <v>8214.72</v>
       </c>
       <c r="D70" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-143'!D$4:D$10,'PA-LEG-143'!$C$4:$C$10,"Google",'PA-LEG-143'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-143'!D$4:D$10,'HD-143'!$C$4:$C$10,"Google",'HD-143'!$B$4:$B$10,"R")</f>
         <v>8214.72</v>
       </c>
       <c r="E70" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-143'!D$4:D$10,'PA-LEG-143'!$C$4:$C$10,"Google",'PA-LEG-143'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-143'!D$4:D$10,'HD-143'!$C$4:$C$10,"Google",'HD-143'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F70" s="5" t="n">
@@ -3328,15 +3328,15 @@
         <v>10</v>
       </c>
       <c r="C71" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-143'!D$4:D$10,'PA-LEG-143'!$C$4:$C$10,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-143'!D$4:D$10,'HD-143'!$C$4:$C$10,"Facebook")</f>
         <v>1325.59</v>
       </c>
       <c r="D71" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-143'!D$4:D$10,'PA-LEG-143'!$C$4:$C$10,"Facebook",'PA-LEG-143'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-143'!D$4:D$10,'HD-143'!$C$4:$C$10,"Facebook",'HD-143'!$B$4:$B$10,"R")</f>
         <v>1325.59</v>
       </c>
       <c r="E71" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-143'!D$4:D$10,'PA-LEG-143'!$C$4:$C$10,"Facebook",'PA-LEG-143'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-143'!D$4:D$10,'HD-143'!$C$4:$C$10,"Facebook",'HD-143'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F71" s="5" t="n">
@@ -3350,11 +3350,11 @@
         <v>11</v>
       </c>
       <c r="C72" s="7" t="n">
-        <f aca="false">'PA-LEG-143'!D10</f>
+        <f aca="false">'HD-143'!D10</f>
         <v>9540.31</v>
       </c>
       <c r="D72" s="7" t="n">
-        <f aca="false">'PA-LEG-143'!D8</f>
+        <f aca="false">'HD-143'!D8</f>
         <v>9540.31</v>
       </c>
       <c r="E72" s="7" t="n">
@@ -3374,15 +3374,15 @@
         <v>8</v>
       </c>
       <c r="C74" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-144'!D$4:D$24,'PA-LEG-144'!$C$4:$C$24,"CTV")</f>
+        <f aca="false">SUMIFS('HD-144'!D$4:D$24,'HD-144'!$C$4:$C$24,"CTV")</f>
         <v>1448.29</v>
       </c>
       <c r="D74" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-144'!D$4:D$24,'PA-LEG-144'!$C$4:$C$24,"CTV",'PA-LEG-144'!$B$4:$B$24,"R")</f>
+        <f aca="false">SUMIFS('HD-144'!D$4:D$24,'HD-144'!$C$4:$C$24,"CTV",'HD-144'!$B$4:$B$24,"R")</f>
         <v>0</v>
       </c>
       <c r="E74" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-144'!D$4:D$24,'PA-LEG-144'!$C$4:$C$24,"CTV",'PA-LEG-144'!$B$4:$B$24,"D")</f>
+        <f aca="false">SUMIFS('HD-144'!D$4:D$24,'HD-144'!$C$4:$C$24,"CTV",'HD-144'!$B$4:$B$24,"D")</f>
         <v>1448.29</v>
       </c>
       <c r="F74" s="5" t="n">
@@ -3396,15 +3396,15 @@
         <v>9</v>
       </c>
       <c r="C75" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-144'!D$4:D$24,'PA-LEG-144'!$C$4:$C$24,"Google")</f>
+        <f aca="false">SUMIFS('HD-144'!D$4:D$24,'HD-144'!$C$4:$C$24,"Google")</f>
         <v>10764.7</v>
       </c>
       <c r="D75" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-144'!D$4:D$24,'PA-LEG-144'!$C$4:$C$24,"Google",'PA-LEG-144'!$B$4:$B$24,"R")</f>
+        <f aca="false">SUMIFS('HD-144'!D$4:D$24,'HD-144'!$C$4:$C$24,"Google",'HD-144'!$B$4:$B$24,"R")</f>
         <v>9464.7</v>
       </c>
       <c r="E75" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-144'!D$4:D$24,'PA-LEG-144'!$C$4:$C$24,"Google",'PA-LEG-144'!$B$4:$B$24,"D")</f>
+        <f aca="false">SUMIFS('HD-144'!D$4:D$24,'HD-144'!$C$4:$C$24,"Google",'HD-144'!$B$4:$B$24,"D")</f>
         <v>1300</v>
       </c>
       <c r="F75" s="5" t="n">
@@ -3418,15 +3418,15 @@
         <v>10</v>
       </c>
       <c r="C76" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-144'!D$4:D$24,'PA-LEG-144'!$C$4:$C$24,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-144'!D$4:D$24,'HD-144'!$C$4:$C$24,"Facebook")</f>
         <v>2019.66</v>
       </c>
       <c r="D76" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-144'!D$4:D$24,'PA-LEG-144'!$C$4:$C$24,"Facebook",'PA-LEG-144'!$B$4:$B$24,"R")</f>
+        <f aca="false">SUMIFS('HD-144'!D$4:D$24,'HD-144'!$C$4:$C$24,"Facebook",'HD-144'!$B$4:$B$24,"R")</f>
         <v>772.85</v>
       </c>
       <c r="E76" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-144'!D$4:D$24,'PA-LEG-144'!$C$4:$C$24,"Facebook",'PA-LEG-144'!$B$4:$B$24,"D")</f>
+        <f aca="false">SUMIFS('HD-144'!D$4:D$24,'HD-144'!$C$4:$C$24,"Facebook",'HD-144'!$B$4:$B$24,"D")</f>
         <v>1246.81</v>
       </c>
       <c r="F76" s="5" t="n">
@@ -3440,15 +3440,15 @@
         <v>11</v>
       </c>
       <c r="C77" s="7" t="n">
-        <f aca="false">'PA-LEG-144'!D24</f>
+        <f aca="false">'HD-144'!D24</f>
         <v>14232.65</v>
       </c>
       <c r="D77" s="7" t="n">
-        <f aca="false">'PA-LEG-144'!D8</f>
+        <f aca="false">'HD-144'!D8</f>
         <v>10237.55</v>
       </c>
       <c r="E77" s="7" t="n">
-        <f aca="false">'PA-LEG-144'!D22</f>
+        <f aca="false">'HD-144'!D22</f>
         <v>3995.1</v>
       </c>
       <c r="F77" s="7" t="n">
@@ -3464,15 +3464,15 @@
         <v>8</v>
       </c>
       <c r="C79" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-147'!D$4:D$10,'PA-LEG-147'!$C$4:$C$10,"CTV")</f>
+        <f aca="false">SUMIFS('HD-147'!D$4:D$10,'HD-147'!$C$4:$C$10,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D79" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-147'!D$4:D$10,'PA-LEG-147'!$C$4:$C$10,"CTV",'PA-LEG-147'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-147'!D$4:D$10,'HD-147'!$C$4:$C$10,"CTV",'HD-147'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E79" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-147'!D$4:D$10,'PA-LEG-147'!$C$4:$C$10,"CTV",'PA-LEG-147'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-147'!D$4:D$10,'HD-147'!$C$4:$C$10,"CTV",'HD-147'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F79" s="5" t="n">
@@ -3486,15 +3486,15 @@
         <v>9</v>
       </c>
       <c r="C80" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-147'!D$4:D$10,'PA-LEG-147'!$C$4:$C$10,"Google")</f>
+        <f aca="false">SUMIFS('HD-147'!D$4:D$10,'HD-147'!$C$4:$C$10,"Google")</f>
         <v>9688.93</v>
       </c>
       <c r="D80" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-147'!D$4:D$10,'PA-LEG-147'!$C$4:$C$10,"Google",'PA-LEG-147'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-147'!D$4:D$10,'HD-147'!$C$4:$C$10,"Google",'HD-147'!$B$4:$B$10,"R")</f>
         <v>9688.93</v>
       </c>
       <c r="E80" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-147'!D$4:D$10,'PA-LEG-147'!$C$4:$C$10,"Google",'PA-LEG-147'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-147'!D$4:D$10,'HD-147'!$C$4:$C$10,"Google",'HD-147'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F80" s="5" t="n">
@@ -3508,15 +3508,15 @@
         <v>10</v>
       </c>
       <c r="C81" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-147'!D$4:D$10,'PA-LEG-147'!$C$4:$C$10,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-147'!D$4:D$10,'HD-147'!$C$4:$C$10,"Facebook")</f>
         <v>1283.57</v>
       </c>
       <c r="D81" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-147'!D$4:D$10,'PA-LEG-147'!$C$4:$C$10,"Facebook",'PA-LEG-147'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-147'!D$4:D$10,'HD-147'!$C$4:$C$10,"Facebook",'HD-147'!$B$4:$B$10,"R")</f>
         <v>1283.57</v>
       </c>
       <c r="E81" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-147'!D$4:D$10,'PA-LEG-147'!$C$4:$C$10,"Facebook",'PA-LEG-147'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-147'!D$4:D$10,'HD-147'!$C$4:$C$10,"Facebook",'HD-147'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F81" s="5" t="n">
@@ -3530,11 +3530,11 @@
         <v>11</v>
       </c>
       <c r="C82" s="7" t="n">
-        <f aca="false">'PA-LEG-147'!D10</f>
+        <f aca="false">'HD-147'!D10</f>
         <v>10972.5</v>
       </c>
       <c r="D82" s="7" t="n">
-        <f aca="false">'PA-LEG-147'!D8</f>
+        <f aca="false">'HD-147'!D8</f>
         <v>10972.5</v>
       </c>
       <c r="E82" s="7" t="n">
@@ -3554,15 +3554,15 @@
         <v>8</v>
       </c>
       <c r="C84" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-160'!D$4:D$23,'PA-LEG-160'!$C$4:$C$23,"CTV")</f>
+        <f aca="false">SUMIFS('HD-160'!D$4:D$23,'HD-160'!$C$4:$C$23,"CTV")</f>
         <v>2845.33</v>
       </c>
       <c r="D84" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-160'!D$4:D$23,'PA-LEG-160'!$C$4:$C$23,"CTV",'PA-LEG-160'!$B$4:$B$23,"R")</f>
+        <f aca="false">SUMIFS('HD-160'!D$4:D$23,'HD-160'!$C$4:$C$23,"CTV",'HD-160'!$B$4:$B$23,"R")</f>
         <v>0</v>
       </c>
       <c r="E84" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-160'!D$4:D$23,'PA-LEG-160'!$C$4:$C$23,"CTV",'PA-LEG-160'!$B$4:$B$23,"D")</f>
+        <f aca="false">SUMIFS('HD-160'!D$4:D$23,'HD-160'!$C$4:$C$23,"CTV",'HD-160'!$B$4:$B$23,"D")</f>
         <v>2845.33</v>
       </c>
       <c r="F84" s="5" t="n">
@@ -3576,15 +3576,15 @@
         <v>9</v>
       </c>
       <c r="C85" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-160'!D$4:D$23,'PA-LEG-160'!$C$4:$C$23,"Google")</f>
+        <f aca="false">SUMIFS('HD-160'!D$4:D$23,'HD-160'!$C$4:$C$23,"Google")</f>
         <v>18233.9</v>
       </c>
       <c r="D85" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-160'!D$4:D$23,'PA-LEG-160'!$C$4:$C$23,"Google",'PA-LEG-160'!$B$4:$B$23,"R")</f>
+        <f aca="false">SUMIFS('HD-160'!D$4:D$23,'HD-160'!$C$4:$C$23,"Google",'HD-160'!$B$4:$B$23,"R")</f>
         <v>10229.48</v>
       </c>
       <c r="E85" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-160'!D$4:D$23,'PA-LEG-160'!$C$4:$C$23,"Google",'PA-LEG-160'!$B$4:$B$23,"D")</f>
+        <f aca="false">SUMIFS('HD-160'!D$4:D$23,'HD-160'!$C$4:$C$23,"Google",'HD-160'!$B$4:$B$23,"D")</f>
         <v>8004.42</v>
       </c>
       <c r="F85" s="5" t="n">
@@ -3598,15 +3598,15 @@
         <v>10</v>
       </c>
       <c r="C86" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-160'!D$4:D$23,'PA-LEG-160'!$C$4:$C$23,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-160'!D$4:D$23,'HD-160'!$C$4:$C$23,"Facebook")</f>
         <v>4042.35</v>
       </c>
       <c r="D86" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-160'!D$4:D$23,'PA-LEG-160'!$C$4:$C$23,"Facebook",'PA-LEG-160'!$B$4:$B$23,"R")</f>
+        <f aca="false">SUMIFS('HD-160'!D$4:D$23,'HD-160'!$C$4:$C$23,"Facebook",'HD-160'!$B$4:$B$23,"R")</f>
         <v>1790.8</v>
       </c>
       <c r="E86" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-160'!D$4:D$23,'PA-LEG-160'!$C$4:$C$23,"Facebook",'PA-LEG-160'!$B$4:$B$23,"D")</f>
+        <f aca="false">SUMIFS('HD-160'!D$4:D$23,'HD-160'!$C$4:$C$23,"Facebook",'HD-160'!$B$4:$B$23,"D")</f>
         <v>2251.55</v>
       </c>
       <c r="F86" s="5" t="n">
@@ -3620,15 +3620,15 @@
         <v>11</v>
       </c>
       <c r="C87" s="7" t="n">
-        <f aca="false">'PA-LEG-160'!D23</f>
+        <f aca="false">'HD-160'!D23</f>
         <v>25121.58</v>
       </c>
       <c r="D87" s="7" t="n">
-        <f aca="false">'PA-LEG-160'!D11</f>
+        <f aca="false">'HD-160'!D11</f>
         <v>12020.28</v>
       </c>
       <c r="E87" s="7" t="n">
-        <f aca="false">'PA-LEG-160'!D21</f>
+        <f aca="false">'HD-160'!D21</f>
         <v>13101.3</v>
       </c>
       <c r="F87" s="7" t="n">
@@ -3644,15 +3644,15 @@
         <v>8</v>
       </c>
       <c r="C89" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-170'!D$4:D$13,'PA-LEG-170'!$C$4:$C$13,"CTV")</f>
+        <f aca="false">SUMIFS('HD-170'!D$4:D$13,'HD-170'!$C$4:$C$13,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D89" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-170'!D$4:D$13,'PA-LEG-170'!$C$4:$C$13,"CTV",'PA-LEG-170'!$B$4:$B$13,"R")</f>
+        <f aca="false">SUMIFS('HD-170'!D$4:D$13,'HD-170'!$C$4:$C$13,"CTV",'HD-170'!$B$4:$B$13,"R")</f>
         <v>0</v>
       </c>
       <c r="E89" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-170'!D$4:D$13,'PA-LEG-170'!$C$4:$C$13,"CTV",'PA-LEG-170'!$B$4:$B$13,"D")</f>
+        <f aca="false">SUMIFS('HD-170'!D$4:D$13,'HD-170'!$C$4:$C$13,"CTV",'HD-170'!$B$4:$B$13,"D")</f>
         <v>0</v>
       </c>
       <c r="F89" s="5" t="n">
@@ -3666,15 +3666,15 @@
         <v>9</v>
       </c>
       <c r="C90" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-170'!D$4:D$13,'PA-LEG-170'!$C$4:$C$13,"Google")</f>
+        <f aca="false">SUMIFS('HD-170'!D$4:D$13,'HD-170'!$C$4:$C$13,"Google")</f>
         <v>9577.31</v>
       </c>
       <c r="D90" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-170'!D$4:D$13,'PA-LEG-170'!$C$4:$C$13,"Google",'PA-LEG-170'!$B$4:$B$13,"R")</f>
+        <f aca="false">SUMIFS('HD-170'!D$4:D$13,'HD-170'!$C$4:$C$13,"Google",'HD-170'!$B$4:$B$13,"R")</f>
         <v>9577.31</v>
       </c>
       <c r="E90" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-170'!D$4:D$13,'PA-LEG-170'!$C$4:$C$13,"Google",'PA-LEG-170'!$B$4:$B$13,"D")</f>
+        <f aca="false">SUMIFS('HD-170'!D$4:D$13,'HD-170'!$C$4:$C$13,"Google",'HD-170'!$B$4:$B$13,"D")</f>
         <v>0</v>
       </c>
       <c r="F90" s="5" t="n">
@@ -3688,15 +3688,15 @@
         <v>10</v>
       </c>
       <c r="C91" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-170'!D$4:D$13,'PA-LEG-170'!$C$4:$C$13,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-170'!D$4:D$13,'HD-170'!$C$4:$C$13,"Facebook")</f>
         <v>2431.81</v>
       </c>
       <c r="D91" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-170'!D$4:D$13,'PA-LEG-170'!$C$4:$C$13,"Facebook",'PA-LEG-170'!$B$4:$B$13,"R")</f>
+        <f aca="false">SUMIFS('HD-170'!D$4:D$13,'HD-170'!$C$4:$C$13,"Facebook",'HD-170'!$B$4:$B$13,"R")</f>
         <v>2431.81</v>
       </c>
       <c r="E91" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-170'!D$4:D$13,'PA-LEG-170'!$C$4:$C$13,"Facebook",'PA-LEG-170'!$B$4:$B$13,"D")</f>
+        <f aca="false">SUMIFS('HD-170'!D$4:D$13,'HD-170'!$C$4:$C$13,"Facebook",'HD-170'!$B$4:$B$13,"D")</f>
         <v>0</v>
       </c>
       <c r="F91" s="5" t="n">
@@ -3710,11 +3710,11 @@
         <v>11</v>
       </c>
       <c r="C92" s="7" t="n">
-        <f aca="false">'PA-LEG-170'!D13</f>
+        <f aca="false">'HD-170'!D13</f>
         <v>12009.12</v>
       </c>
       <c r="D92" s="7" t="n">
-        <f aca="false">'PA-LEG-170'!D11</f>
+        <f aca="false">'HD-170'!D11</f>
         <v>12009.12</v>
       </c>
       <c r="E92" s="7" t="n">
@@ -3734,15 +3734,15 @@
         <v>8</v>
       </c>
       <c r="C94" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-187'!D$4:D$10,'PA-LEG-187'!$C$4:$C$10,"CTV")</f>
+        <f aca="false">SUMIFS('HD-187'!D$4:D$10,'HD-187'!$C$4:$C$10,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D94" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-187'!D$4:D$10,'PA-LEG-187'!$C$4:$C$10,"CTV",'PA-LEG-187'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-187'!D$4:D$10,'HD-187'!$C$4:$C$10,"CTV",'HD-187'!$B$4:$B$10,"R")</f>
         <v>0</v>
       </c>
       <c r="E94" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-187'!D$4:D$10,'PA-LEG-187'!$C$4:$C$10,"CTV",'PA-LEG-187'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-187'!D$4:D$10,'HD-187'!$C$4:$C$10,"CTV",'HD-187'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F94" s="5" t="n">
@@ -3756,15 +3756,15 @@
         <v>9</v>
       </c>
       <c r="C95" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-187'!D$4:D$10,'PA-LEG-187'!$C$4:$C$10,"Google")</f>
+        <f aca="false">SUMIFS('HD-187'!D$4:D$10,'HD-187'!$C$4:$C$10,"Google")</f>
         <v>9832.05</v>
       </c>
       <c r="D95" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-187'!D$4:D$10,'PA-LEG-187'!$C$4:$C$10,"Google",'PA-LEG-187'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-187'!D$4:D$10,'HD-187'!$C$4:$C$10,"Google",'HD-187'!$B$4:$B$10,"R")</f>
         <v>9832.05</v>
       </c>
       <c r="E95" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-187'!D$4:D$10,'PA-LEG-187'!$C$4:$C$10,"Google",'PA-LEG-187'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-187'!D$4:D$10,'HD-187'!$C$4:$C$10,"Google",'HD-187'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F95" s="5" t="n">
@@ -3778,15 +3778,15 @@
         <v>10</v>
       </c>
       <c r="C96" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-187'!D$4:D$10,'PA-LEG-187'!$C$4:$C$10,"Facebook")</f>
+        <f aca="false">SUMIFS('HD-187'!D$4:D$10,'HD-187'!$C$4:$C$10,"Facebook")</f>
         <v>1239.99</v>
       </c>
       <c r="D96" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-187'!D$4:D$10,'PA-LEG-187'!$C$4:$C$10,"Facebook",'PA-LEG-187'!$B$4:$B$10,"R")</f>
+        <f aca="false">SUMIFS('HD-187'!D$4:D$10,'HD-187'!$C$4:$C$10,"Facebook",'HD-187'!$B$4:$B$10,"R")</f>
         <v>1239.99</v>
       </c>
       <c r="E96" s="5" t="n">
-        <f aca="false">SUMIFS('PA-LEG-187'!D$4:D$10,'PA-LEG-187'!$C$4:$C$10,"Facebook",'PA-LEG-187'!$B$4:$B$10,"D")</f>
+        <f aca="false">SUMIFS('HD-187'!D$4:D$10,'HD-187'!$C$4:$C$10,"Facebook",'HD-187'!$B$4:$B$10,"D")</f>
         <v>0</v>
       </c>
       <c r="F96" s="5" t="n">
@@ -3800,11 +3800,11 @@
         <v>11</v>
       </c>
       <c r="C97" s="7" t="n">
-        <f aca="false">'PA-LEG-187'!D10</f>
+        <f aca="false">'HD-187'!D10</f>
         <v>11072.04</v>
       </c>
       <c r="D97" s="7" t="n">
-        <f aca="false">'PA-LEG-187'!D8</f>
+        <f aca="false">'HD-187'!D8</f>
         <v>11072.04</v>
       </c>
       <c r="E97" s="7" t="n">
@@ -3824,15 +3824,15 @@
         <v>8</v>
       </c>
       <c r="C99" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-06'!D$4:D$20,'PA-STSEN-06'!$C$4:$C$20,"CTV")</f>
+        <f aca="false">SUMIFS('SD-6'!D$4:D$20,'SD-6'!$C$4:$C$20,"CTV")</f>
         <v>9.04</v>
       </c>
       <c r="D99" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-06'!D$4:D$20,'PA-STSEN-06'!$C$4:$C$20,"CTV",'PA-STSEN-06'!$B$4:$B$20,"R")</f>
+        <f aca="false">SUMIFS('SD-6'!D$4:D$20,'SD-6'!$C$4:$C$20,"CTV",'SD-6'!$B$4:$B$20,"R")</f>
         <v>9.04</v>
       </c>
       <c r="E99" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-06'!D$4:D$20,'PA-STSEN-06'!$C$4:$C$20,"CTV",'PA-STSEN-06'!$B$4:$B$20,"D")</f>
+        <f aca="false">SUMIFS('SD-6'!D$4:D$20,'SD-6'!$C$4:$C$20,"CTV",'SD-6'!$B$4:$B$20,"D")</f>
         <v>0</v>
       </c>
       <c r="F99" s="5" t="n">
@@ -3846,15 +3846,15 @@
         <v>9</v>
       </c>
       <c r="C100" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-06'!D$4:D$20,'PA-STSEN-06'!$C$4:$C$20,"Google")</f>
+        <f aca="false">SUMIFS('SD-6'!D$4:D$20,'SD-6'!$C$4:$C$20,"Google")</f>
         <v>35578.2</v>
       </c>
       <c r="D100" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-06'!D$4:D$20,'PA-STSEN-06'!$C$4:$C$20,"Google",'PA-STSEN-06'!$B$4:$B$20,"R")</f>
+        <f aca="false">SUMIFS('SD-6'!D$4:D$20,'SD-6'!$C$4:$C$20,"Google",'SD-6'!$B$4:$B$20,"R")</f>
         <v>35578.2</v>
       </c>
       <c r="E100" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-06'!D$4:D$20,'PA-STSEN-06'!$C$4:$C$20,"Google",'PA-STSEN-06'!$B$4:$B$20,"D")</f>
+        <f aca="false">SUMIFS('SD-6'!D$4:D$20,'SD-6'!$C$4:$C$20,"Google",'SD-6'!$B$4:$B$20,"D")</f>
         <v>0</v>
       </c>
       <c r="F100" s="5" t="n">
@@ -3868,15 +3868,15 @@
         <v>10</v>
       </c>
       <c r="C101" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-06'!D$4:D$20,'PA-STSEN-06'!$C$4:$C$20,"Facebook")</f>
+        <f aca="false">SUMIFS('SD-6'!D$4:D$20,'SD-6'!$C$4:$C$20,"Facebook")</f>
         <v>57192.31</v>
       </c>
       <c r="D101" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-06'!D$4:D$20,'PA-STSEN-06'!$C$4:$C$20,"Facebook",'PA-STSEN-06'!$B$4:$B$20,"R")</f>
+        <f aca="false">SUMIFS('SD-6'!D$4:D$20,'SD-6'!$C$4:$C$20,"Facebook",'SD-6'!$B$4:$B$20,"R")</f>
         <v>33435.24</v>
       </c>
       <c r="E101" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-06'!D$4:D$20,'PA-STSEN-06'!$C$4:$C$20,"Facebook",'PA-STSEN-06'!$B$4:$B$20,"D")</f>
+        <f aca="false">SUMIFS('SD-6'!D$4:D$20,'SD-6'!$C$4:$C$20,"Facebook",'SD-6'!$B$4:$B$20,"D")</f>
         <v>23757.07</v>
       </c>
       <c r="F101" s="5" t="n">
@@ -3890,15 +3890,15 @@
         <v>11</v>
       </c>
       <c r="C102" s="7" t="n">
-        <f aca="false">'PA-STSEN-06'!D20</f>
+        <f aca="false">'SD-6'!D20</f>
         <v>92779.55</v>
       </c>
       <c r="D102" s="7" t="n">
-        <f aca="false">'PA-STSEN-06'!D13</f>
+        <f aca="false">'SD-6'!D13</f>
         <v>69022.48</v>
       </c>
       <c r="E102" s="7" t="n">
-        <f aca="false">'PA-STSEN-06'!D18</f>
+        <f aca="false">'SD-6'!D18</f>
         <v>23757.07</v>
       </c>
       <c r="F102" s="7" t="n">
@@ -3914,15 +3914,15 @@
         <v>8</v>
       </c>
       <c r="C104" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-16'!D$4:D$20,'PA-STSEN-16'!$C$4:$C$20,"CTV")</f>
+        <f aca="false">SUMIFS('SD-16'!D$4:D$20,'SD-16'!$C$4:$C$20,"CTV")</f>
         <v>2940.77</v>
       </c>
       <c r="D104" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-16'!D$4:D$20,'PA-STSEN-16'!$C$4:$C$20,"CTV",'PA-STSEN-16'!$B$4:$B$20,"R")</f>
+        <f aca="false">SUMIFS('SD-16'!D$4:D$20,'SD-16'!$C$4:$C$20,"CTV",'SD-16'!$B$4:$B$20,"R")</f>
         <v>2940.77</v>
       </c>
       <c r="E104" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-16'!D$4:D$20,'PA-STSEN-16'!$C$4:$C$20,"CTV",'PA-STSEN-16'!$B$4:$B$20,"D")</f>
+        <f aca="false">SUMIFS('SD-16'!D$4:D$20,'SD-16'!$C$4:$C$20,"CTV",'SD-16'!$B$4:$B$20,"D")</f>
         <v>0</v>
       </c>
       <c r="F104" s="5" t="n">
@@ -3936,15 +3936,15 @@
         <v>9</v>
       </c>
       <c r="C105" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-16'!D$4:D$20,'PA-STSEN-16'!$C$4:$C$20,"Google")</f>
+        <f aca="false">SUMIFS('SD-16'!D$4:D$20,'SD-16'!$C$4:$C$20,"Google")</f>
         <v>55373.74</v>
       </c>
       <c r="D105" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-16'!D$4:D$20,'PA-STSEN-16'!$C$4:$C$20,"Google",'PA-STSEN-16'!$B$4:$B$20,"R")</f>
+        <f aca="false">SUMIFS('SD-16'!D$4:D$20,'SD-16'!$C$4:$C$20,"Google",'SD-16'!$B$4:$B$20,"R")</f>
         <v>51832.11</v>
       </c>
       <c r="E105" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-16'!D$4:D$20,'PA-STSEN-16'!$C$4:$C$20,"Google",'PA-STSEN-16'!$B$4:$B$20,"D")</f>
+        <f aca="false">SUMIFS('SD-16'!D$4:D$20,'SD-16'!$C$4:$C$20,"Google",'SD-16'!$B$4:$B$20,"D")</f>
         <v>3541.63</v>
       </c>
       <c r="F105" s="5" t="n">
@@ -3958,15 +3958,15 @@
         <v>10</v>
       </c>
       <c r="C106" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-16'!D$4:D$20,'PA-STSEN-16'!$C$4:$C$20,"Facebook")</f>
+        <f aca="false">SUMIFS('SD-16'!D$4:D$20,'SD-16'!$C$4:$C$20,"Facebook")</f>
         <v>28759.66</v>
       </c>
       <c r="D106" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-16'!D$4:D$20,'PA-STSEN-16'!$C$4:$C$20,"Facebook",'PA-STSEN-16'!$B$4:$B$20,"R")</f>
+        <f aca="false">SUMIFS('SD-16'!D$4:D$20,'SD-16'!$C$4:$C$20,"Facebook",'SD-16'!$B$4:$B$20,"R")</f>
         <v>4687.92</v>
       </c>
       <c r="E106" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-16'!D$4:D$20,'PA-STSEN-16'!$C$4:$C$20,"Facebook",'PA-STSEN-16'!$B$4:$B$20,"D")</f>
+        <f aca="false">SUMIFS('SD-16'!D$4:D$20,'SD-16'!$C$4:$C$20,"Facebook",'SD-16'!$B$4:$B$20,"D")</f>
         <v>24071.74</v>
       </c>
       <c r="F106" s="5" t="n">
@@ -3980,15 +3980,15 @@
         <v>11</v>
       </c>
       <c r="C107" s="7" t="n">
-        <f aca="false">'PA-STSEN-16'!D20</f>
+        <f aca="false">'SD-16'!D20</f>
         <v>87074.17</v>
       </c>
       <c r="D107" s="7" t="n">
-        <f aca="false">'PA-STSEN-16'!D12</f>
+        <f aca="false">'SD-16'!D12</f>
         <v>59460.8</v>
       </c>
       <c r="E107" s="7" t="n">
-        <f aca="false">'PA-STSEN-16'!D18</f>
+        <f aca="false">'SD-16'!D18</f>
         <v>27613.37</v>
       </c>
       <c r="F107" s="7" t="n">
@@ -4004,15 +4004,15 @@
         <v>8</v>
       </c>
       <c r="C109" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-24'!D$4:D$25,'PA-STSEN-24'!$C$4:$C$25,"CTV")</f>
+        <f aca="false">SUMIFS('SD-24'!D$4:D$25,'SD-24'!$C$4:$C$25,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D109" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-24'!D$4:D$25,'PA-STSEN-24'!$C$4:$C$25,"CTV",'PA-STSEN-24'!$B$4:$B$25,"R")</f>
+        <f aca="false">SUMIFS('SD-24'!D$4:D$25,'SD-24'!$C$4:$C$25,"CTV",'SD-24'!$B$4:$B$25,"R")</f>
         <v>0</v>
       </c>
       <c r="E109" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-24'!D$4:D$25,'PA-STSEN-24'!$C$4:$C$25,"CTV",'PA-STSEN-24'!$B$4:$B$25,"D")</f>
+        <f aca="false">SUMIFS('SD-24'!D$4:D$25,'SD-24'!$C$4:$C$25,"CTV",'SD-24'!$B$4:$B$25,"D")</f>
         <v>0</v>
       </c>
       <c r="F109" s="5" t="n">
@@ -4026,15 +4026,15 @@
         <v>9</v>
       </c>
       <c r="C110" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-24'!D$4:D$25,'PA-STSEN-24'!$C$4:$C$25,"Google")</f>
+        <f aca="false">SUMIFS('SD-24'!D$4:D$25,'SD-24'!$C$4:$C$25,"Google")</f>
         <v>36743.78</v>
       </c>
       <c r="D110" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-24'!D$4:D$25,'PA-STSEN-24'!$C$4:$C$25,"Google",'PA-STSEN-24'!$B$4:$B$25,"R")</f>
+        <f aca="false">SUMIFS('SD-24'!D$4:D$25,'SD-24'!$C$4:$C$25,"Google",'SD-24'!$B$4:$B$25,"R")</f>
         <v>26543.78</v>
       </c>
       <c r="E110" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-24'!D$4:D$25,'PA-STSEN-24'!$C$4:$C$25,"Google",'PA-STSEN-24'!$B$4:$B$25,"D")</f>
+        <f aca="false">SUMIFS('SD-24'!D$4:D$25,'SD-24'!$C$4:$C$25,"Google",'SD-24'!$B$4:$B$25,"D")</f>
         <v>10200</v>
       </c>
       <c r="F110" s="5" t="n">
@@ -4048,15 +4048,15 @@
         <v>10</v>
       </c>
       <c r="C111" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-24'!D$4:D$25,'PA-STSEN-24'!$C$4:$C$25,"Facebook")</f>
+        <f aca="false">SUMIFS('SD-24'!D$4:D$25,'SD-24'!$C$4:$C$25,"Facebook")</f>
         <v>68589.02</v>
       </c>
       <c r="D111" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-24'!D$4:D$25,'PA-STSEN-24'!$C$4:$C$25,"Facebook",'PA-STSEN-24'!$B$4:$B$25,"R")</f>
+        <f aca="false">SUMIFS('SD-24'!D$4:D$25,'SD-24'!$C$4:$C$25,"Facebook",'SD-24'!$B$4:$B$25,"R")</f>
         <v>32931.78</v>
       </c>
       <c r="E111" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-24'!D$4:D$25,'PA-STSEN-24'!$C$4:$C$25,"Facebook",'PA-STSEN-24'!$B$4:$B$25,"D")</f>
+        <f aca="false">SUMIFS('SD-24'!D$4:D$25,'SD-24'!$C$4:$C$25,"Facebook",'SD-24'!$B$4:$B$25,"D")</f>
         <v>35657.24</v>
       </c>
       <c r="F111" s="5" t="n">
@@ -4070,15 +4070,15 @@
         <v>11</v>
       </c>
       <c r="C112" s="7" t="n">
-        <f aca="false">'PA-STSEN-24'!D25</f>
+        <f aca="false">'SD-24'!D25</f>
         <v>105332.8</v>
       </c>
       <c r="D112" s="7" t="n">
-        <f aca="false">'PA-STSEN-24'!D14</f>
+        <f aca="false">'SD-24'!D14</f>
         <v>59475.56</v>
       </c>
       <c r="E112" s="7" t="n">
-        <f aca="false">'PA-STSEN-24'!D23</f>
+        <f aca="false">'SD-24'!D23</f>
         <v>45857.24</v>
       </c>
       <c r="F112" s="7" t="n">
@@ -4094,15 +4094,15 @@
         <v>8</v>
       </c>
       <c r="C114" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-40'!D$4:D$20,'PA-STSEN-40'!$C$4:$C$20,"CTV")</f>
+        <f aca="false">SUMIFS('SD-40'!D$4:D$20,'SD-40'!$C$4:$C$20,"CTV")</f>
         <v>0</v>
       </c>
       <c r="D114" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-40'!D$4:D$20,'PA-STSEN-40'!$C$4:$C$20,"CTV",'PA-STSEN-40'!$B$4:$B$20,"R")</f>
+        <f aca="false">SUMIFS('SD-40'!D$4:D$20,'SD-40'!$C$4:$C$20,"CTV",'SD-40'!$B$4:$B$20,"R")</f>
         <v>0</v>
       </c>
       <c r="E114" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-40'!D$4:D$20,'PA-STSEN-40'!$C$4:$C$20,"CTV",'PA-STSEN-40'!$B$4:$B$20,"D")</f>
+        <f aca="false">SUMIFS('SD-40'!D$4:D$20,'SD-40'!$C$4:$C$20,"CTV",'SD-40'!$B$4:$B$20,"D")</f>
         <v>0</v>
       </c>
       <c r="F114" s="5" t="n">
@@ -4116,15 +4116,15 @@
         <v>9</v>
       </c>
       <c r="C115" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-40'!D$4:D$20,'PA-STSEN-40'!$C$4:$C$20,"Google")</f>
+        <f aca="false">SUMIFS('SD-40'!D$4:D$20,'SD-40'!$C$4:$C$20,"Google")</f>
         <v>37949.08</v>
       </c>
       <c r="D115" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-40'!D$4:D$20,'PA-STSEN-40'!$C$4:$C$20,"Google",'PA-STSEN-40'!$B$4:$B$20,"R")</f>
+        <f aca="false">SUMIFS('SD-40'!D$4:D$20,'SD-40'!$C$4:$C$20,"Google",'SD-40'!$B$4:$B$20,"R")</f>
         <v>34879.67</v>
       </c>
       <c r="E115" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-40'!D$4:D$20,'PA-STSEN-40'!$C$4:$C$20,"Google",'PA-STSEN-40'!$B$4:$B$20,"D")</f>
+        <f aca="false">SUMIFS('SD-40'!D$4:D$20,'SD-40'!$C$4:$C$20,"Google",'SD-40'!$B$4:$B$20,"D")</f>
         <v>3069.41</v>
       </c>
       <c r="F115" s="5" t="n">
@@ -4138,15 +4138,15 @@
         <v>10</v>
       </c>
       <c r="C116" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-40'!D$4:D$20,'PA-STSEN-40'!$C$4:$C$20,"Facebook")</f>
+        <f aca="false">SUMIFS('SD-40'!D$4:D$20,'SD-40'!$C$4:$C$20,"Facebook")</f>
         <v>34853.09</v>
       </c>
       <c r="D116" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-40'!D$4:D$20,'PA-STSEN-40'!$C$4:$C$20,"Facebook",'PA-STSEN-40'!$B$4:$B$20,"R")</f>
+        <f aca="false">SUMIFS('SD-40'!D$4:D$20,'SD-40'!$C$4:$C$20,"Facebook",'SD-40'!$B$4:$B$20,"R")</f>
         <v>10878.67</v>
       </c>
       <c r="E116" s="5" t="n">
-        <f aca="false">SUMIFS('PA-STSEN-40'!D$4:D$20,'PA-STSEN-40'!$C$4:$C$20,"Facebook",'PA-STSEN-40'!$B$4:$B$20,"D")</f>
+        <f aca="false">SUMIFS('SD-40'!D$4:D$20,'SD-40'!$C$4:$C$20,"Facebook",'SD-40'!$B$4:$B$20,"D")</f>
         <v>23974.42</v>
       </c>
       <c r="F116" s="5" t="n">
@@ -4160,15 +4160,15 @@
         <v>11</v>
       </c>
       <c r="C117" s="7" t="n">
-        <f aca="false">'PA-STSEN-40'!D20</f>
+        <f aca="false">'SD-40'!D20</f>
         <v>72802.17</v>
       </c>
       <c r="D117" s="7" t="n">
-        <f aca="false">'PA-STSEN-40'!D12</f>
+        <f aca="false">'SD-40'!D12</f>
         <v>45758.34</v>
       </c>
       <c r="E117" s="7" t="n">
-        <f aca="false">'PA-STSEN-40'!D18</f>
+        <f aca="false">'SD-40'!D18</f>
         <v>27043.83</v>
       </c>
       <c r="F117" s="7" t="n">
@@ -4250,29 +4250,29 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="A4" r:id="rId1" location="'PA-LEG-13'!A1" display="State House District 13"/>
-    <hyperlink ref="A9" r:id="rId2" location="'PA-LEG-16'!A1" display="State House District 16"/>
-    <hyperlink ref="A14" r:id="rId3" location="'PA-LEG-18'!A1" display="State House District 18"/>
-    <hyperlink ref="A19" r:id="rId4" location="'PA-LEG-28'!A1" display="State House District 28"/>
-    <hyperlink ref="A24" r:id="rId5" location="'PA-LEG-41'!A1" display="State House District 41"/>
-    <hyperlink ref="A29" r:id="rId6" location="'PA-LEG-44'!A1" display="State House District 44"/>
-    <hyperlink ref="A34" r:id="rId7" location="'PA-LEG-46'!A1" display="State House District 46"/>
-    <hyperlink ref="A39" r:id="rId8" location="'PA-LEG-72'!A1" display="State House District 72"/>
-    <hyperlink ref="A44" r:id="rId9" location="'PA-LEG-88'!A1" display="State House District 88"/>
-    <hyperlink ref="A49" r:id="rId10" location="'PA-LEG-118'!A1" display="State House District 118"/>
-    <hyperlink ref="A54" r:id="rId11" location="'PA-LEG-121'!A1" display="State House District 121"/>
-    <hyperlink ref="A59" r:id="rId12" location="'PA-LEG-137'!A1" display="State House District 137"/>
-    <hyperlink ref="A64" r:id="rId13" location="'PA-LEG-142'!A1" display="State House District 142"/>
-    <hyperlink ref="A69" r:id="rId14" location="'PA-LEG-143'!A1" display="State House District 143"/>
-    <hyperlink ref="A74" r:id="rId15" location="'PA-LEG-144'!A1" display="State House District 144"/>
-    <hyperlink ref="A79" r:id="rId16" location="'PA-LEG-147'!A1" display="State House District 147"/>
-    <hyperlink ref="A84" r:id="rId17" location="'PA-LEG-160'!A1" display="State House District 160"/>
-    <hyperlink ref="A89" r:id="rId18" location="'PA-LEG-170'!A1" display="State House District 170"/>
-    <hyperlink ref="A94" r:id="rId19" location="'PA-LEG-187'!A1" display="State House District 187"/>
-    <hyperlink ref="A99" r:id="rId20" location="'PA-STSEN-06'!A1" display="State Senate District 6"/>
-    <hyperlink ref="A104" r:id="rId21" location="'PA-STSEN-16'!A1" display="State Senate District 16"/>
-    <hyperlink ref="A109" r:id="rId22" location="'PA-STSEN-24'!A1" display="State Senate District 24"/>
-    <hyperlink ref="A114" r:id="rId23" location="'PA-STSEN-40'!A1" display="State Senate District 40"/>
+    <hyperlink ref="A4" r:id="rId1" location="'HD-13'!A1" display="State House District 13"/>
+    <hyperlink ref="A9" r:id="rId2" location="'HD-16'!A1" display="State House District 16"/>
+    <hyperlink ref="A14" r:id="rId3" location="'HD-18'!A1" display="State House District 18"/>
+    <hyperlink ref="A19" r:id="rId4" location="'HD-28'!A1" display="State House District 28"/>
+    <hyperlink ref="A24" r:id="rId5" location="'HD-41'!A1" display="State House District 41"/>
+    <hyperlink ref="A29" r:id="rId6" location="'HD-44'!A1" display="State House District 44"/>
+    <hyperlink ref="A34" r:id="rId7" location="'HD-46'!A1" display="State House District 46"/>
+    <hyperlink ref="A39" r:id="rId8" location="'HD-72'!A1" display="State House District 72"/>
+    <hyperlink ref="A44" r:id="rId9" location="'HD-88'!A1" display="State House District 88"/>
+    <hyperlink ref="A49" r:id="rId10" location="'HD-118'!A1" display="State House District 118"/>
+    <hyperlink ref="A54" r:id="rId11" location="'HD-121'!A1" display="State House District 121"/>
+    <hyperlink ref="A59" r:id="rId12" location="'HD-137'!A1" display="State House District 137"/>
+    <hyperlink ref="A64" r:id="rId13" location="'HD-142'!A1" display="State House District 142"/>
+    <hyperlink ref="A69" r:id="rId14" location="'HD-143'!A1" display="State House District 143"/>
+    <hyperlink ref="A74" r:id="rId15" location="'HD-144'!A1" display="State House District 144"/>
+    <hyperlink ref="A79" r:id="rId16" location="'HD-147'!A1" display="State House District 147"/>
+    <hyperlink ref="A84" r:id="rId17" location="'HD-160'!A1" display="State House District 160"/>
+    <hyperlink ref="A89" r:id="rId18" location="'HD-170'!A1" display="State House District 170"/>
+    <hyperlink ref="A94" r:id="rId19" location="'HD-187'!A1" display="State House District 187"/>
+    <hyperlink ref="A99" r:id="rId20" location="'SD-6'!A1" display="State Senate District 6"/>
+    <hyperlink ref="A104" r:id="rId21" location="'SD-16'!A1" display="State Senate District 16"/>
+    <hyperlink ref="A109" r:id="rId22" location="'SD-24'!A1" display="State Senate District 24"/>
+    <hyperlink ref="A114" r:id="rId23" location="'SD-40'!A1" display="State Senate District 40"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Match race tab headers to the new HD/SD tab names
The in-sheet navy header now shows the same abbreviated name as the
tab itself (e.g. "HD-13"), instead of the old raw race code — no more
mismatch between what you click and what you land on.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MLDJZYpWcKSroEnjKzk6cV
</commit_message>
<xml_diff>
--- a/reports/PA_Digital_Competitive_Report.xlsx
+++ b/reports/PA_Digital_Competitive_Report.xlsx
@@ -179,7 +179,7 @@
     <t xml:space="preserve">Report prepared by GPS Impact  |  Confidential</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-13</t>
+    <t xml:space="preserve">HD-13</t>
   </si>
   <si>
     <t xml:space="preserve">CANDIDATE / COMMITTEE</t>
@@ -236,7 +236,7 @@
     <t xml:space="preserve">GRAND TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-16</t>
+    <t xml:space="preserve">HD-16</t>
   </si>
   <si>
     <t xml:space="preserve">ROB MATZIE STATE HOUSE</t>
@@ -257,7 +257,7 @@
     <t xml:space="preserve">DEMOCRAT PARTY TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-18</t>
+    <t xml:space="preserve">HD-18</t>
   </si>
   <si>
     <t xml:space="preserve">BETTER PA</t>
@@ -266,13 +266,13 @@
     <t xml:space="preserve">BETTER PA Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-28</t>
+    <t xml:space="preserve">HD-28</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-41</t>
+    <t xml:space="preserve">HD-41</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-44</t>
+    <t xml:space="preserve">HD-44</t>
   </si>
   <si>
     <t xml:space="preserve">HADLEY HAAS STATE HOUSE</t>
@@ -287,7 +287,7 @@
     <t xml:space="preserve">FAIR DEMOCRACY Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-46</t>
+    <t xml:space="preserve">HD-46</t>
   </si>
   <si>
     <t xml:space="preserve">JASON ORTITAY STATE HOUSE</t>
@@ -296,7 +296,7 @@
     <t xml:space="preserve">JASON ORTITAY STATE HOUSE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-72</t>
+    <t xml:space="preserve">HD-72</t>
   </si>
   <si>
     <t xml:space="preserve">CITIZENS ALLIANCE PA</t>
@@ -317,7 +317,7 @@
     <t xml:space="preserve">NEA Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-88</t>
+    <t xml:space="preserve">HD-88</t>
   </si>
   <si>
     <t xml:space="preserve">SARA AGERTON STATE HOUSE</t>
@@ -326,7 +326,7 @@
     <t xml:space="preserve">SARA AGERTON STATE HOUSE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-118</t>
+    <t xml:space="preserve">HD-118</t>
   </si>
   <si>
     <t xml:space="preserve">JIM HADDOCK STATE HOUSE</t>
@@ -335,7 +335,7 @@
     <t xml:space="preserve">JIM HADDOCK STATE HOUSE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-121</t>
+    <t xml:space="preserve">HD-121</t>
   </si>
   <si>
     <t xml:space="preserve">JESSICA MCCLAY STATE HOUSE</t>
@@ -344,7 +344,7 @@
     <t xml:space="preserve">JESSICA MCCLAY STATE HOUSE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-137</t>
+    <t xml:space="preserve">HD-137</t>
   </si>
   <si>
     <t xml:space="preserve">JOE EMRICK STATE HOUSE</t>
@@ -353,7 +353,7 @@
     <t xml:space="preserve">JOE EMRICK STATE HOUSE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-142</t>
+    <t xml:space="preserve">HD-142</t>
   </si>
   <si>
     <t xml:space="preserve">KRISTIN EGAN STATE HOUSE</t>
@@ -362,10 +362,10 @@
     <t xml:space="preserve">KRISTIN EGAN STATE HOUSE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-143</t>
+    <t xml:space="preserve">HD-143</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-144</t>
+    <t xml:space="preserve">HD-144</t>
   </si>
   <si>
     <t xml:space="preserve">BRIAN MUNROE STATE HOUSE</t>
@@ -380,10 +380,10 @@
     <t xml:space="preserve">PA HDCC Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-147</t>
+    <t xml:space="preserve">HD-147</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-160</t>
+    <t xml:space="preserve">HD-160</t>
   </si>
   <si>
     <t xml:space="preserve">CRAIG WILLIAMS STATE HOUSE</t>
@@ -392,7 +392,7 @@
     <t xml:space="preserve">CRAIG WILLIAMS STATE HOUSE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-170</t>
+    <t xml:space="preserve">HD-170</t>
   </si>
   <si>
     <t xml:space="preserve">MARTINA WHITE STATE HOUSE</t>
@@ -401,10 +401,10 @@
     <t xml:space="preserve">MARTINA WHITE STATE HOUSE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-LEG-187</t>
+    <t xml:space="preserve">HD-187</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-STSEN-06</t>
+    <t xml:space="preserve">SD-6</t>
   </si>
   <si>
     <t xml:space="preserve">FRANK FARRY STATE SENATE</t>
@@ -413,7 +413,7 @@
     <t xml:space="preserve">FRANK FARRY STATE SENATE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-STSEN-16</t>
+    <t xml:space="preserve">SD-16</t>
   </si>
   <si>
     <t xml:space="preserve">JARRETT COLEMAN STATE SENATE</t>
@@ -422,7 +422,7 @@
     <t xml:space="preserve">JARRETT COLEMAN STATE SENATE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-STSEN-24</t>
+    <t xml:space="preserve">SD-24</t>
   </si>
   <si>
     <t xml:space="preserve">TRACY PENNYCUICK STATE SENATE</t>
@@ -443,7 +443,7 @@
     <t xml:space="preserve">CHRIS THOMAS STATE SENATE Total</t>
   </si>
   <si>
-    <t xml:space="preserve">PA-STSEN-40</t>
+    <t xml:space="preserve">SD-40</t>
   </si>
   <si>
     <t xml:space="preserve">ROSEMARY BROWN STATE SENATE</t>

</xml_diff>

<commit_message>
Fix Summary hyperlinks so they don't break when the file moves
Assigning a plain string to cell.hyperlink makes openpyxl store it as
an external link target, even when the string starts with "#" — it
gets written as a real relationship (TargetMode="External") pointing
at that literal string. Excel resolves external hyperlinks relative
to wherever the workbook was first saved, so as soon as the file was
downloaded/moved anywhere else, clicking a district name tried to
open a path that no longer existed.

Fixed by constructing the Hyperlink object explicitly with
location=... instead, which openpyxl writes as a same-workbook
reference with no relationship at all. Confirmed in the raw XML: the
hyperlink now carries only a location attribute, and the sheet's only
relationship is for the logo image.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MLDJZYpWcKSroEnjKzk6cV
</commit_message>
<xml_diff>
--- a/reports/PA_Digital_Competitive_Report.xlsx
+++ b/reports/PA_Digital_Competitive_Report.xlsx
@@ -4250,29 +4250,29 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="A4" r:id="rId1" location="'HD-13'!A1" display="State House District 13"/>
-    <hyperlink ref="A9" r:id="rId2" location="'HD-16'!A1" display="State House District 16"/>
-    <hyperlink ref="A14" r:id="rId3" location="'HD-18'!A1" display="State House District 18"/>
-    <hyperlink ref="A19" r:id="rId4" location="'HD-28'!A1" display="State House District 28"/>
-    <hyperlink ref="A24" r:id="rId5" location="'HD-41'!A1" display="State House District 41"/>
-    <hyperlink ref="A29" r:id="rId6" location="'HD-44'!A1" display="State House District 44"/>
-    <hyperlink ref="A34" r:id="rId7" location="'HD-46'!A1" display="State House District 46"/>
-    <hyperlink ref="A39" r:id="rId8" location="'HD-72'!A1" display="State House District 72"/>
-    <hyperlink ref="A44" r:id="rId9" location="'HD-88'!A1" display="State House District 88"/>
-    <hyperlink ref="A49" r:id="rId10" location="'HD-118'!A1" display="State House District 118"/>
-    <hyperlink ref="A54" r:id="rId11" location="'HD-121'!A1" display="State House District 121"/>
-    <hyperlink ref="A59" r:id="rId12" location="'HD-137'!A1" display="State House District 137"/>
-    <hyperlink ref="A64" r:id="rId13" location="'HD-142'!A1" display="State House District 142"/>
-    <hyperlink ref="A69" r:id="rId14" location="'HD-143'!A1" display="State House District 143"/>
-    <hyperlink ref="A74" r:id="rId15" location="'HD-144'!A1" display="State House District 144"/>
-    <hyperlink ref="A79" r:id="rId16" location="'HD-147'!A1" display="State House District 147"/>
-    <hyperlink ref="A84" r:id="rId17" location="'HD-160'!A1" display="State House District 160"/>
-    <hyperlink ref="A89" r:id="rId18" location="'HD-170'!A1" display="State House District 170"/>
-    <hyperlink ref="A94" r:id="rId19" location="'HD-187'!A1" display="State House District 187"/>
-    <hyperlink ref="A99" r:id="rId20" location="'SD-6'!A1" display="State Senate District 6"/>
-    <hyperlink ref="A104" r:id="rId21" location="'SD-16'!A1" display="State Senate District 16"/>
-    <hyperlink ref="A109" r:id="rId22" location="'SD-24'!A1" display="State Senate District 24"/>
-    <hyperlink ref="A114" r:id="rId23" location="'SD-40'!A1" display="State Senate District 40"/>
+    <hyperlink ref="A4" location="'HD-13'!A1" display="State House District 13"/>
+    <hyperlink ref="A9" location="'HD-16'!A1" display="State House District 16"/>
+    <hyperlink ref="A14" location="'HD-18'!A1" display="State House District 18"/>
+    <hyperlink ref="A19" location="'HD-28'!A1" display="State House District 28"/>
+    <hyperlink ref="A24" location="'HD-41'!A1" display="State House District 41"/>
+    <hyperlink ref="A29" location="'HD-44'!A1" display="State House District 44"/>
+    <hyperlink ref="A34" location="'HD-46'!A1" display="State House District 46"/>
+    <hyperlink ref="A39" location="'HD-72'!A1" display="State House District 72"/>
+    <hyperlink ref="A44" location="'HD-88'!A1" display="State House District 88"/>
+    <hyperlink ref="A49" location="'HD-118'!A1" display="State House District 118"/>
+    <hyperlink ref="A54" location="'HD-121'!A1" display="State House District 121"/>
+    <hyperlink ref="A59" location="'HD-137'!A1" display="State House District 137"/>
+    <hyperlink ref="A64" location="'HD-142'!A1" display="State House District 142"/>
+    <hyperlink ref="A69" location="'HD-143'!A1" display="State House District 143"/>
+    <hyperlink ref="A74" location="'HD-144'!A1" display="State House District 144"/>
+    <hyperlink ref="A79" location="'HD-147'!A1" display="State House District 147"/>
+    <hyperlink ref="A84" location="'HD-160'!A1" display="State House District 160"/>
+    <hyperlink ref="A89" location="'HD-170'!A1" display="State House District 170"/>
+    <hyperlink ref="A94" location="'HD-187'!A1" display="State House District 187"/>
+    <hyperlink ref="A99" location="'SD-6'!A1" display="State Senate District 6"/>
+    <hyperlink ref="A104" location="'SD-16'!A1" display="State Senate District 16"/>
+    <hyperlink ref="A109" location="'SD-24'!A1" display="State Senate District 24"/>
+    <hyperlink ref="A114" location="'SD-40'!A1" display="State Senate District 40"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4281,7 +4281,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId24"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>